<commit_message>
Fix trading signal system: resolve duplicates, correct distance formatting, and improve telegram report sorting
- Remove duplicate stock entries by eliminating data persistence logic
- Fix Excel percentage formatting (0.00% -> 0.00%%) to display correct values
- Add distance-based sorting in telegram reports (lowest distance first)
- Maintain 10% alert threshold and group priority (buy approach -> bought -> sell approach)
- Ensure trading_signals.xlsx contains only current analysis results (not cumulative)
</commit_message>
<xml_diff>
--- a/output/turnover_universe.xlsx
+++ b/output/turnover_universe.xlsx
@@ -9,16 +9,15 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="universe" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="165" formatCode="000000"/>
-    <numFmt numFmtId="166" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -142,7 +141,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -151,6 +150,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -162,25 +164,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -199,18 +193,6 @@
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -572,7 +554,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H67"/>
+  <dimension ref="A1:H70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -584,1470 +566,1695 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="13" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>첫주도주</t>
         </is>
       </c>
-      <c r="B1" s="13" t="inlineStr">
+      <c r="B1" s="10" t="inlineStr">
         <is>
           <t>최근주도주</t>
         </is>
       </c>
-      <c r="C1" s="13" t="inlineStr">
+      <c r="C1" s="10" t="inlineStr">
         <is>
           <t>티커</t>
         </is>
       </c>
-      <c r="D1" s="13" t="inlineStr">
+      <c r="D1" s="10" t="inlineStr">
         <is>
           <t>종목명</t>
         </is>
       </c>
-      <c r="E1" s="13" t="inlineStr">
+      <c r="E1" s="10" t="inlineStr">
         <is>
           <t>거래대금(억)</t>
         </is>
       </c>
-      <c r="F1" s="13" t="inlineStr">
+      <c r="F1" s="10" t="inlineStr">
         <is>
           <t>누적횟수</t>
         </is>
       </c>
-      <c r="H1" s="14" t="inlineStr">
-        <is>
-          <t>최종 업데이트: 2025-10-15</t>
+      <c r="H1" s="11" t="inlineStr">
+        <is>
+          <t>최종 업데이트: 2025-10-17</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="15" t="n">
+      <c r="A2" s="12" t="n">
         <v>45942</v>
       </c>
-      <c r="B2" s="15" t="n">
+      <c r="B2" s="12" t="n">
+        <v>45947</v>
+      </c>
+      <c r="C2" s="13" t="inlineStr">
+        <is>
+          <t>005930</t>
+        </is>
+      </c>
+      <c r="D2" s="14" t="inlineStr">
+        <is>
+          <t>삼성전자</t>
+        </is>
+      </c>
+      <c r="E2" s="15" t="n">
+        <v>24723.21</v>
+      </c>
+      <c r="F2" s="16" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="n">
+        <v>45942</v>
+      </c>
+      <c r="B3" s="12" t="n">
+        <v>45947</v>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>000660</t>
+        </is>
+      </c>
+      <c r="D3" s="14" t="inlineStr">
+        <is>
+          <t>SK하이닉스</t>
+        </is>
+      </c>
+      <c r="E3" s="15" t="n">
+        <v>22464.63</v>
+      </c>
+      <c r="F3" s="16" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="n">
+        <v>45942</v>
+      </c>
+      <c r="B4" s="12" t="n">
+        <v>45947</v>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>034020</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>두산에너빌리티</t>
+        </is>
+      </c>
+      <c r="E4" s="15" t="n">
+        <v>8415.57</v>
+      </c>
+      <c r="F4" s="16" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="n">
+        <v>45942</v>
+      </c>
+      <c r="B5" s="12" t="n">
         <v>45945</v>
       </c>
-      <c r="C2" s="16" t="inlineStr">
-        <is>
-          <t>005930</t>
-        </is>
-      </c>
-      <c r="D2" s="17" t="inlineStr">
-        <is>
-          <t>삼성전자</t>
-        </is>
-      </c>
-      <c r="E2" s="18" t="n">
-        <v>32197.17</v>
-      </c>
-      <c r="F2" s="19" t="n">
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>035420</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>NAVER</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="n">
+        <v>5570.25</v>
+      </c>
+      <c r="F5" s="16" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="15" t="n">
+    <row r="6">
+      <c r="A6" s="12" t="n">
         <v>45942</v>
       </c>
-      <c r="B3" s="15" t="n">
+      <c r="B6" s="12" t="n">
         <v>45945</v>
       </c>
-      <c r="C3" s="16" t="inlineStr">
-        <is>
-          <t>000660</t>
-        </is>
-      </c>
-      <c r="D3" s="17" t="inlineStr">
-        <is>
-          <t>SK하이닉스</t>
-        </is>
-      </c>
-      <c r="E3" s="18" t="n">
-        <v>16787.64</v>
-      </c>
-      <c r="F3" s="19" t="n">
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>042700</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>한미반도체</t>
+        </is>
+      </c>
+      <c r="E6" s="15" t="n">
+        <v>10101.19</v>
+      </c>
+      <c r="F6" s="16" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="15" t="n">
+    <row r="7">
+      <c r="A7" s="12" t="n">
+        <v>45874</v>
+      </c>
+      <c r="B7" s="12" t="n">
+        <v>45947</v>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>247540</t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>에코프로비엠</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="n">
+        <v>11340.85</v>
+      </c>
+      <c r="F7" s="16" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="n">
+        <v>45730</v>
+      </c>
+      <c r="B8" s="12" t="n">
+        <v>45947</v>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>006400</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>삼성SDI</t>
+        </is>
+      </c>
+      <c r="E8" s="15" t="n">
+        <v>7189.43</v>
+      </c>
+      <c r="F8" s="16" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="n">
+        <v>45916</v>
+      </c>
+      <c r="B9" s="12" t="n">
+        <v>45945</v>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>125490</t>
+        </is>
+      </c>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>한라캐스트</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="n">
+        <v>5614.12</v>
+      </c>
+      <c r="F9" s="16" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="n">
+        <v>45947</v>
+      </c>
+      <c r="B10" s="12" t="n">
+        <v>45947</v>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>086520</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>에코프로</t>
+        </is>
+      </c>
+      <c r="E10" s="15" t="n">
+        <v>13280.34</v>
+      </c>
+      <c r="F10" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="n">
+        <v>45947</v>
+      </c>
+      <c r="B11" s="12" t="n">
+        <v>45947</v>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>450080</t>
+        </is>
+      </c>
+      <c r="D11" s="14" t="inlineStr">
+        <is>
+          <t>에코프로머티</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="n">
+        <v>5520.35</v>
+      </c>
+      <c r="F11" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="n">
+        <v>45946</v>
+      </c>
+      <c r="B12" s="12" t="n">
+        <v>45946</v>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>373220</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>LG에너지솔루션</t>
+        </is>
+      </c>
+      <c r="E12" s="15" t="n">
+        <v>41700</v>
+      </c>
+      <c r="F12" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="n">
+        <v>45943</v>
+      </c>
+      <c r="B13" s="12" t="n">
+        <v>45943</v>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>466100</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>클로봇</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="n">
+        <v>6494.860000000001</v>
+      </c>
+      <c r="F13" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="n">
         <v>45942</v>
       </c>
-      <c r="B4" s="15" t="n">
-        <v>45945</v>
-      </c>
-      <c r="C4" s="16" t="inlineStr">
-        <is>
-          <t>034020</t>
-        </is>
-      </c>
-      <c r="D4" s="17" t="inlineStr">
-        <is>
-          <t>두산에너빌리티</t>
-        </is>
-      </c>
-      <c r="E4" s="18" t="n">
-        <v>22662.65</v>
-      </c>
-      <c r="F4" s="19" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="15" t="n">
+      <c r="B14" s="12" t="n">
         <v>45942</v>
       </c>
-      <c r="B5" s="15" t="n">
-        <v>45945</v>
-      </c>
-      <c r="C5" s="16" t="inlineStr">
-        <is>
-          <t>035420</t>
-        </is>
-      </c>
-      <c r="D5" s="17" t="inlineStr">
-        <is>
-          <t>NAVER</t>
-        </is>
-      </c>
-      <c r="E5" s="18" t="n">
-        <v>5570.25</v>
-      </c>
-      <c r="F5" s="19" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="15" t="n">
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>108490</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>로보티즈</t>
+        </is>
+      </c>
+      <c r="E14" s="15" t="n">
+        <v>8159.77</v>
+      </c>
+      <c r="F14" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="n">
         <v>45942</v>
       </c>
-      <c r="B6" s="15" t="n">
-        <v>45945</v>
-      </c>
-      <c r="C6" s="16" t="inlineStr">
-        <is>
-          <t>042700</t>
-        </is>
-      </c>
-      <c r="D6" s="17" t="inlineStr">
-        <is>
-          <t>한미반도체</t>
-        </is>
-      </c>
-      <c r="E6" s="18" t="n">
-        <v>10101.19</v>
-      </c>
-      <c r="F6" s="19" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="15" t="n">
-        <v>45916</v>
-      </c>
-      <c r="B7" s="15" t="n">
-        <v>45945</v>
-      </c>
-      <c r="C7" s="16" t="inlineStr">
-        <is>
-          <t>125490</t>
-        </is>
-      </c>
-      <c r="D7" s="17" t="inlineStr">
-        <is>
-          <t>한라캐스트</t>
-        </is>
-      </c>
-      <c r="E7" s="18" t="n">
-        <v>5614.12</v>
-      </c>
-      <c r="F7" s="19" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="15" t="n">
-        <v>45943</v>
-      </c>
-      <c r="B8" s="15" t="n">
-        <v>45943</v>
-      </c>
-      <c r="C8" s="16" t="inlineStr">
-        <is>
-          <t>466100</t>
-        </is>
-      </c>
-      <c r="D8" s="17" t="inlineStr">
-        <is>
-          <t>클로봇</t>
-        </is>
-      </c>
-      <c r="E8" s="18" t="n">
-        <v>6494.860000000001</v>
-      </c>
-      <c r="F8" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="15" t="n">
+      <c r="B15" s="12" t="n">
         <v>45942</v>
       </c>
-      <c r="B9" s="15" t="n">
-        <v>45942</v>
-      </c>
-      <c r="C9" s="16" t="inlineStr">
-        <is>
-          <t>108490</t>
-        </is>
-      </c>
-      <c r="D9" s="17" t="inlineStr">
-        <is>
-          <t>로보티즈</t>
-        </is>
-      </c>
-      <c r="E9" s="18" t="n">
-        <v>8159.77</v>
-      </c>
-      <c r="F9" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="15" t="n">
-        <v>45942</v>
-      </c>
-      <c r="B10" s="15" t="n">
-        <v>45942</v>
-      </c>
-      <c r="C10" s="16" t="inlineStr">
+      <c r="C15" s="13" t="inlineStr">
         <is>
           <t>005935</t>
         </is>
       </c>
-      <c r="D10" s="17" t="inlineStr">
+      <c r="D15" s="14" t="inlineStr">
         <is>
           <t>삼성전자우</t>
         </is>
       </c>
-      <c r="E10" s="18" t="n">
+      <c r="E15" s="15" t="n">
         <v>5438.03</v>
       </c>
-      <c r="F10" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="15" t="n">
+      <c r="F15" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="n">
         <v>44512</v>
       </c>
-      <c r="B11" s="15" t="n">
+      <c r="B16" s="12" t="n">
         <v>45929</v>
       </c>
-      <c r="C11" s="16" t="inlineStr">
+      <c r="C16" s="13" t="inlineStr">
         <is>
           <t>249420</t>
         </is>
       </c>
-      <c r="D11" s="17" t="inlineStr">
+      <c r="D16" s="14" t="inlineStr">
         <is>
           <t>일동제약</t>
         </is>
       </c>
-      <c r="E11" s="18" t="n">
+      <c r="E16" s="15" t="n">
         <v>9183</v>
       </c>
-      <c r="F11" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="15" t="n">
+      <c r="F16" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="n">
         <v>45849</v>
       </c>
-      <c r="B12" s="15" t="n">
+      <c r="B17" s="12" t="n">
         <v>45929</v>
       </c>
-      <c r="C12" s="16" t="inlineStr">
+      <c r="C17" s="13" t="inlineStr">
         <is>
           <t>041190</t>
         </is>
       </c>
-      <c r="D12" s="17" t="inlineStr">
+      <c r="D17" s="14" t="inlineStr">
         <is>
           <t>우리기술투자</t>
         </is>
       </c>
-      <c r="E12" s="18" t="n">
+      <c r="E17" s="15" t="n">
         <v>5517</v>
       </c>
-      <c r="F12" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="15" t="n">
+      <c r="F17" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="n">
         <v>45849</v>
       </c>
-      <c r="B13" s="15" t="n">
+      <c r="B18" s="12" t="n">
         <v>45926</v>
       </c>
-      <c r="C13" s="16" t="inlineStr">
+      <c r="C18" s="13" t="inlineStr">
         <is>
           <t>060250</t>
         </is>
       </c>
-      <c r="D13" s="17" t="inlineStr">
+      <c r="D18" s="14" t="inlineStr">
         <is>
           <t>NHN KCP</t>
         </is>
       </c>
-      <c r="E13" s="18" t="n">
+      <c r="E18" s="15" t="n">
         <v>9171</v>
       </c>
-      <c r="F13" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="15" t="n">
+      <c r="F18" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="n">
         <v>44876</v>
       </c>
-      <c r="B14" s="15" t="n">
+      <c r="B19" s="12" t="n">
         <v>45926</v>
       </c>
-      <c r="C14" s="16" t="inlineStr">
+      <c r="C19" s="13" t="inlineStr">
         <is>
           <t>035720</t>
         </is>
       </c>
-      <c r="D14" s="17" t="inlineStr">
+      <c r="D19" s="14" t="inlineStr">
         <is>
           <t>카카오</t>
         </is>
       </c>
-      <c r="E14" s="18" t="n">
+      <c r="E19" s="15" t="n">
         <v>5080</v>
       </c>
-      <c r="F14" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="15" t="n">
+      <c r="F19" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="n">
         <v>45925</v>
       </c>
-      <c r="B15" s="15" t="n">
+      <c r="B20" s="12" t="n">
         <v>45925</v>
       </c>
-      <c r="C15" s="16" t="inlineStr">
+      <c r="C20" s="13" t="inlineStr">
         <is>
           <t>277810</t>
         </is>
       </c>
-      <c r="D15" s="17" t="inlineStr">
+      <c r="D20" s="14" t="inlineStr">
         <is>
           <t>레인보우로보틱스</t>
         </is>
       </c>
-      <c r="E15" s="18" t="n">
+      <c r="E20" s="15" t="n">
         <v>7211</v>
       </c>
-      <c r="F15" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="15" t="n">
+      <c r="F20" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="n">
         <v>45650</v>
       </c>
-      <c r="B16" s="15" t="n">
+      <c r="B21" s="12" t="n">
         <v>45924</v>
       </c>
-      <c r="C16" s="16" t="inlineStr">
+      <c r="C21" s="13" t="inlineStr">
         <is>
           <t>196170</t>
         </is>
       </c>
-      <c r="D16" s="17" t="inlineStr">
+      <c r="D21" s="14" t="inlineStr">
         <is>
           <t>알테오젠</t>
         </is>
       </c>
-      <c r="E16" s="18" t="n">
+      <c r="E21" s="15" t="n">
         <v>5188</v>
       </c>
-      <c r="F16" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="15" t="n">
+      <c r="F21" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="n">
         <v>44515</v>
       </c>
-      <c r="B17" s="15" t="n">
+      <c r="B22" s="12" t="n">
         <v>45923</v>
       </c>
-      <c r="C17" s="16" t="inlineStr">
+      <c r="C22" s="13" t="inlineStr">
         <is>
           <t>068270</t>
         </is>
       </c>
-      <c r="D17" s="17" t="inlineStr">
+      <c r="D22" s="14" t="inlineStr">
         <is>
           <t>셀트리온</t>
         </is>
       </c>
-      <c r="F17" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="15" t="n">
+      <c r="E22" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F22" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="n">
         <v>45922</v>
       </c>
-      <c r="B18" s="15" t="n">
+      <c r="B23" s="12" t="n">
         <v>45923</v>
       </c>
-      <c r="C18" s="16" t="inlineStr">
+      <c r="C23" s="13" t="inlineStr">
         <is>
           <t>347850</t>
         </is>
       </c>
-      <c r="D18" s="17" t="inlineStr">
+      <c r="D23" s="14" t="inlineStr">
         <is>
           <t>디앤디파마텍</t>
         </is>
       </c>
-      <c r="F18" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="15" t="n">
+      <c r="E23" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F23" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="n">
         <v>45377</v>
       </c>
-      <c r="B19" s="15" t="n">
+      <c r="B24" s="12" t="n">
         <v>45919</v>
       </c>
-      <c r="C19" s="16" t="inlineStr">
+      <c r="C24" s="13" t="inlineStr">
         <is>
           <t>000250</t>
         </is>
       </c>
-      <c r="D19" s="17" t="inlineStr">
+      <c r="D24" s="14" t="inlineStr">
         <is>
           <t>삼천당제약</t>
         </is>
       </c>
-      <c r="F19" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="15" t="n">
+      <c r="E24" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F24" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="n">
         <v>45839</v>
       </c>
-      <c r="B20" s="15" t="n">
+      <c r="B25" s="12" t="n">
         <v>45919</v>
       </c>
-      <c r="C20" s="16" t="inlineStr">
+      <c r="C25" s="13" t="inlineStr">
         <is>
           <t>064260</t>
         </is>
       </c>
-      <c r="D20" s="17" t="inlineStr">
+      <c r="D25" s="14" t="inlineStr">
         <is>
           <t>다날</t>
         </is>
       </c>
-      <c r="F20" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="15" t="n">
+      <c r="E25" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F25" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="n">
         <v>45694</v>
       </c>
-      <c r="B21" s="15" t="n">
+      <c r="B26" s="12" t="n">
         <v>45919</v>
       </c>
-      <c r="C21" s="16" t="inlineStr">
+      <c r="C26" s="13" t="inlineStr">
         <is>
           <t>064350</t>
         </is>
       </c>
-      <c r="D21" s="17" t="inlineStr">
+      <c r="D26" s="14" t="inlineStr">
         <is>
           <t>현대로템</t>
         </is>
       </c>
-      <c r="F21" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="15" t="n">
+      <c r="E26" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F26" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="n">
         <v>45918</v>
       </c>
-      <c r="B22" s="15" t="n">
+      <c r="B27" s="12" t="n">
         <v>45919</v>
       </c>
-      <c r="C22" s="16" t="inlineStr">
+      <c r="C27" s="13" t="inlineStr">
         <is>
           <t>090360</t>
         </is>
       </c>
-      <c r="D22" s="17" t="inlineStr">
+      <c r="D27" s="14" t="inlineStr">
         <is>
           <t>로보스타</t>
         </is>
       </c>
-      <c r="F22" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="15" t="n">
+      <c r="E27" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F27" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="n">
         <v>45708</v>
       </c>
-      <c r="B23" s="15" t="n">
+      <c r="B28" s="12" t="n">
         <v>45919</v>
       </c>
-      <c r="C23" s="16" t="inlineStr">
+      <c r="C28" s="13" t="inlineStr">
         <is>
           <t>047810</t>
         </is>
       </c>
-      <c r="D23" s="17" t="inlineStr">
+      <c r="D28" s="14" t="inlineStr">
         <is>
           <t>한국항공우주</t>
         </is>
       </c>
-      <c r="F23" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="15" t="n">
+      <c r="E28" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F28" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="n">
         <v>45604</v>
       </c>
-      <c r="B24" s="15" t="n">
+      <c r="B29" s="12" t="n">
         <v>45917</v>
       </c>
-      <c r="C24" s="16" t="inlineStr">
+      <c r="C29" s="13" t="inlineStr">
         <is>
           <t>042660</t>
         </is>
       </c>
-      <c r="D24" s="17" t="inlineStr">
+      <c r="D29" s="14" t="inlineStr">
         <is>
           <t>한화오션</t>
         </is>
       </c>
-      <c r="F24" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="15" t="n">
+      <c r="E29" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F29" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="12" t="n">
         <v>45883</v>
       </c>
-      <c r="B25" s="15" t="n">
+      <c r="B30" s="12" t="n">
         <v>45912</v>
       </c>
-      <c r="C25" s="16" t="inlineStr">
+      <c r="C30" s="13" t="inlineStr">
         <is>
           <t>456160</t>
         </is>
       </c>
-      <c r="D25" s="17" t="inlineStr">
+      <c r="D30" s="14" t="inlineStr">
         <is>
           <t>지투지바이오</t>
         </is>
       </c>
-      <c r="F25" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="15" t="n">
+      <c r="E30" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F30" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="n">
         <v>45912</v>
       </c>
-      <c r="B26" s="15" t="n">
+      <c r="B31" s="12" t="n">
         <v>45912</v>
       </c>
-      <c r="C26" s="16" t="inlineStr">
+      <c r="C31" s="13" t="inlineStr">
         <is>
           <t>004370</t>
         </is>
       </c>
-      <c r="D26" s="17" t="inlineStr">
+      <c r="D31" s="14" t="inlineStr">
         <is>
           <t>농심</t>
         </is>
       </c>
-      <c r="F26" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="15" t="n">
+      <c r="E31" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F31" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="n">
         <v>45911</v>
       </c>
-      <c r="B27" s="15" t="n">
+      <c r="B32" s="12" t="n">
         <v>45912</v>
       </c>
-      <c r="C27" s="16" t="inlineStr">
+      <c r="C32" s="13" t="inlineStr">
         <is>
           <t>100090</t>
         </is>
       </c>
-      <c r="D27" s="17" t="inlineStr">
+      <c r="D32" s="14" t="inlineStr">
         <is>
           <t>SK오션플랜트</t>
         </is>
       </c>
-      <c r="F27" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="15" t="n">
+      <c r="E32" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F32" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="12" t="n">
         <v>45876</v>
       </c>
-      <c r="B28" s="15" t="n">
+      <c r="B33" s="12" t="n">
         <v>45910</v>
       </c>
-      <c r="C28" s="16" t="inlineStr">
+      <c r="C33" s="13" t="inlineStr">
         <is>
           <t>097230</t>
         </is>
       </c>
-      <c r="D28" s="17" t="inlineStr">
+      <c r="D33" s="14" t="inlineStr">
         <is>
           <t>HJ중공업</t>
         </is>
       </c>
-      <c r="F28" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="15" t="n">
+      <c r="E33" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F33" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="12" t="n">
         <v>45908</v>
       </c>
-      <c r="B29" s="15" t="n">
+      <c r="B34" s="12" t="n">
         <v>45910</v>
       </c>
-      <c r="C29" s="16" t="inlineStr">
+      <c r="C34" s="13" t="inlineStr">
         <is>
           <t>075580</t>
         </is>
       </c>
-      <c r="D29" s="17" t="inlineStr">
+      <c r="D34" s="14" t="inlineStr">
         <is>
           <t>세진중공업</t>
         </is>
       </c>
-      <c r="F29" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="15" t="n">
+      <c r="E34" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F34" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="n">
         <v>45908</v>
       </c>
-      <c r="B30" s="15" t="n">
+      <c r="B35" s="12" t="n">
         <v>45908</v>
       </c>
-      <c r="C30" s="16" t="inlineStr">
+      <c r="C35" s="13" t="inlineStr">
         <is>
           <t>290650</t>
         </is>
       </c>
-      <c r="D30" s="17" t="inlineStr">
+      <c r="D35" s="14" t="inlineStr">
         <is>
           <t>엘앤씨바이오</t>
         </is>
       </c>
-      <c r="F30" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="15" t="n">
+      <c r="E35" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F35" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="12" t="n">
         <v>45898</v>
       </c>
-      <c r="B31" s="15" t="n">
+      <c r="B36" s="12" t="n">
         <v>45898</v>
       </c>
-      <c r="C31" s="16" t="inlineStr">
+      <c r="C36" s="13" t="inlineStr">
         <is>
           <t>082740</t>
         </is>
       </c>
-      <c r="D31" s="17" t="inlineStr">
+      <c r="D36" s="14" t="inlineStr">
         <is>
           <t>한화엔진</t>
         </is>
       </c>
-      <c r="F31" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="15" t="n">
+      <c r="E36" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F36" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="12" t="n">
         <v>45897</v>
       </c>
-      <c r="B32" s="15" t="n">
+      <c r="B37" s="12" t="n">
         <v>45897</v>
       </c>
-      <c r="C32" s="16" t="inlineStr">
+      <c r="C37" s="13" t="inlineStr">
         <is>
           <t>460930</t>
         </is>
       </c>
-      <c r="D32" s="17" t="inlineStr">
+      <c r="D37" s="14" t="inlineStr">
         <is>
           <t>현대힘스</t>
         </is>
       </c>
-      <c r="F32" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="15" t="n">
+      <c r="E37" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F37" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="12" t="n">
         <v>45897</v>
       </c>
-      <c r="B33" s="15" t="n">
+      <c r="B38" s="12" t="n">
         <v>45897</v>
       </c>
-      <c r="C33" s="16" t="inlineStr">
+      <c r="C38" s="13" t="inlineStr">
         <is>
           <t>009540</t>
         </is>
       </c>
-      <c r="D33" s="17" t="inlineStr">
+      <c r="D38" s="14" t="inlineStr">
         <is>
           <t>HD한국조선해양</t>
         </is>
       </c>
-      <c r="F33" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="15" t="n">
+      <c r="E38" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F38" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="12" t="n">
         <v>45896</v>
       </c>
-      <c r="B34" s="15" t="n">
+      <c r="B39" s="12" t="n">
         <v>45897</v>
       </c>
-      <c r="C34" s="16" t="inlineStr">
+      <c r="C39" s="13" t="inlineStr">
         <is>
           <t>010620</t>
         </is>
       </c>
-      <c r="D34" s="17" t="inlineStr">
+      <c r="D39" s="14" t="inlineStr">
         <is>
           <t>HD현대미포</t>
         </is>
       </c>
-      <c r="F34" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="15" t="n">
+      <c r="E39" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F39" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="12" t="n">
         <v>45365</v>
       </c>
-      <c r="B35" s="15" t="n">
+      <c r="B40" s="12" t="n">
         <v>45896</v>
       </c>
-      <c r="C35" s="16" t="inlineStr">
+      <c r="C40" s="13" t="inlineStr">
         <is>
           <t>010140</t>
         </is>
       </c>
-      <c r="D35" s="17" t="inlineStr">
+      <c r="D40" s="14" t="inlineStr">
         <is>
           <t>삼성중공업</t>
         </is>
       </c>
-      <c r="F35" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="15" t="n">
+      <c r="E40" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F40" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="12" t="n">
         <v>45895</v>
       </c>
-      <c r="B36" s="15" t="n">
+      <c r="B41" s="12" t="n">
         <v>45895</v>
       </c>
-      <c r="C36" s="16" t="inlineStr">
+      <c r="C41" s="13" t="inlineStr">
         <is>
           <t>298040</t>
         </is>
       </c>
-      <c r="D36" s="17" t="inlineStr">
+      <c r="D41" s="14" t="inlineStr">
         <is>
           <t>효성중공업</t>
         </is>
       </c>
-      <c r="F36" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="15" t="n">
+      <c r="E41" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F41" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="12" t="n">
         <v>45782</v>
       </c>
-      <c r="B37" s="15" t="n">
+      <c r="B42" s="12" t="n">
         <v>45895</v>
       </c>
-      <c r="C37" s="16" t="inlineStr">
+      <c r="C42" s="13" t="inlineStr">
         <is>
           <t>079550</t>
         </is>
       </c>
-      <c r="D37" s="17" t="inlineStr">
+      <c r="D42" s="14" t="inlineStr">
         <is>
           <t>LIG넥스원</t>
         </is>
       </c>
-      <c r="F37" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="15" t="n">
+      <c r="E42" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F42" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="12" t="n">
         <v>45888</v>
       </c>
-      <c r="B38" s="15" t="n">
+      <c r="B43" s="12" t="n">
         <v>45888</v>
       </c>
-      <c r="C38" s="16" t="inlineStr">
-        <is>
-          <t>000080</t>
-        </is>
-      </c>
-      <c r="D38" s="17" t="inlineStr">
+      <c r="C43" s="13" t="inlineStr">
+        <is>
+          <t>0008Z0</t>
+        </is>
+      </c>
+      <c r="D43" s="14" t="inlineStr">
         <is>
           <t>에스엔시스</t>
         </is>
       </c>
-      <c r="F38" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="15" t="n">
+      <c r="E43" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F43" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="12" t="n">
         <v>45887</v>
       </c>
-      <c r="B39" s="15" t="n">
+      <c r="B44" s="12" t="n">
         <v>45887</v>
       </c>
-      <c r="C39" s="16" t="inlineStr">
+      <c r="C44" s="13" t="inlineStr">
         <is>
           <t>484590</t>
         </is>
       </c>
-      <c r="D39" s="17" t="inlineStr">
+      <c r="D44" s="14" t="inlineStr">
         <is>
           <t>삼양컴텍</t>
         </is>
       </c>
-      <c r="F39" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="15" t="n">
+      <c r="E44" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F44" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="12" t="n">
         <v>45755</v>
       </c>
-      <c r="B40" s="15" t="n">
+      <c r="B45" s="12" t="n">
         <v>45883</v>
       </c>
-      <c r="C40" s="16" t="inlineStr">
+      <c r="C45" s="13" t="inlineStr">
         <is>
           <t>298380</t>
         </is>
       </c>
-      <c r="D40" s="17" t="inlineStr">
+      <c r="D45" s="14" t="inlineStr">
         <is>
           <t>에이비엘바이오</t>
         </is>
       </c>
-      <c r="F40" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="15" t="n">
+      <c r="E45" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F45" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="12" t="n">
         <v>45882</v>
       </c>
-      <c r="B41" s="15" t="n">
+      <c r="B46" s="12" t="n">
         <v>45882</v>
       </c>
-      <c r="C41" s="16" t="inlineStr">
+      <c r="C46" s="13" t="inlineStr">
         <is>
           <t>034220</t>
         </is>
       </c>
-      <c r="D41" s="17" t="inlineStr">
+      <c r="D46" s="14" t="inlineStr">
         <is>
           <t>LG디스플레이</t>
         </is>
       </c>
-      <c r="F41" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="15" t="n">
+      <c r="E46" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F46" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="12" t="n">
         <v>45853</v>
       </c>
-      <c r="B42" s="15" t="n">
+      <c r="B47" s="12" t="n">
         <v>45876</v>
       </c>
-      <c r="C42" s="16" t="inlineStr">
+      <c r="C47" s="13" t="inlineStr">
         <is>
           <t>015760</t>
         </is>
       </c>
-      <c r="D42" s="17" t="inlineStr">
+      <c r="D47" s="14" t="inlineStr">
         <is>
           <t>한국전력</t>
         </is>
       </c>
-      <c r="F42" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="15" t="n">
+      <c r="E47" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F47" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="12" t="n">
         <v>45870</v>
       </c>
-      <c r="B43" s="15" t="n">
+      <c r="B48" s="12" t="n">
         <v>45876</v>
       </c>
-      <c r="C43" s="16" t="inlineStr">
+      <c r="C48" s="13" t="inlineStr">
         <is>
           <t>439260</t>
         </is>
       </c>
-      <c r="D43" s="17" t="inlineStr">
+      <c r="D48" s="14" t="inlineStr">
         <is>
           <t>대한조선</t>
         </is>
       </c>
-      <c r="F43" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="15" t="n">
+      <c r="E48" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F48" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="12" t="n">
         <v>45785</v>
       </c>
-      <c r="B44" s="15" t="n">
+      <c r="B49" s="12" t="n">
         <v>45875</v>
       </c>
-      <c r="C44" s="16" t="inlineStr">
+      <c r="C49" s="13" t="inlineStr">
         <is>
           <t>278470</t>
         </is>
       </c>
-      <c r="D44" s="17" t="inlineStr">
+      <c r="D49" s="14" t="inlineStr">
         <is>
           <t>에이피알</t>
         </is>
       </c>
-      <c r="F44" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="15" t="n">
+      <c r="E49" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F49" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="12" t="n">
         <v>45874</v>
       </c>
-      <c r="B45" s="15" t="n">
+      <c r="B50" s="12" t="n">
         <v>45874</v>
       </c>
-      <c r="C45" s="16" t="inlineStr">
+      <c r="C50" s="13" t="inlineStr">
         <is>
           <t>326030</t>
         </is>
       </c>
-      <c r="D45" s="17" t="inlineStr">
+      <c r="D50" s="14" t="inlineStr">
         <is>
           <t>SK바이오팜</t>
         </is>
       </c>
-      <c r="F45" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="15" t="n">
-        <v>45874</v>
-      </c>
-      <c r="B46" s="15" t="n">
-        <v>45874</v>
-      </c>
-      <c r="C46" s="16" t="inlineStr">
-        <is>
-          <t>247540</t>
-        </is>
-      </c>
-      <c r="D46" s="17" t="inlineStr">
-        <is>
-          <t>에코프로비엠</t>
-        </is>
-      </c>
-      <c r="F46" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="15" t="n">
-        <v>45730</v>
-      </c>
-      <c r="B47" s="15" t="n">
-        <v>45874</v>
-      </c>
-      <c r="C47" s="16" t="inlineStr">
-        <is>
-          <t>006400</t>
-        </is>
-      </c>
-      <c r="D47" s="17" t="inlineStr">
-        <is>
-          <t>삼성SDI</t>
-        </is>
-      </c>
-      <c r="F47" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="15" t="n">
+      <c r="E50" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F50" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="12" t="n">
         <v>45699</v>
       </c>
-      <c r="B48" s="15" t="n">
+      <c r="B51" s="12" t="n">
         <v>45870</v>
       </c>
-      <c r="C48" s="16" t="inlineStr">
+      <c r="C51" s="13" t="inlineStr">
         <is>
           <t>012450</t>
         </is>
       </c>
-      <c r="D48" s="17" t="inlineStr">
+      <c r="D51" s="14" t="inlineStr">
         <is>
           <t>한화에어로스페이스</t>
         </is>
       </c>
-      <c r="F48" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="15" t="n">
+      <c r="E51" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F51" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="12" t="n">
         <v>45833</v>
       </c>
-      <c r="B49" s="15" t="n">
+      <c r="B52" s="12" t="n">
         <v>45869</v>
       </c>
-      <c r="C49" s="16" t="inlineStr">
+      <c r="C52" s="13" t="inlineStr">
         <is>
           <t>005380</t>
         </is>
       </c>
-      <c r="D49" s="17" t="inlineStr">
+      <c r="D52" s="14" t="inlineStr">
         <is>
           <t>현대차</t>
         </is>
       </c>
-      <c r="F49" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="15" t="n">
+      <c r="E52" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F52" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="12" t="n">
         <v>45700</v>
       </c>
-      <c r="B50" s="15" t="n">
+      <c r="B53" s="12" t="n">
         <v>45869</v>
       </c>
-      <c r="C50" s="16" t="inlineStr">
+      <c r="C53" s="13" t="inlineStr">
         <is>
           <t>272210</t>
         </is>
       </c>
-      <c r="D50" s="17" t="inlineStr">
+      <c r="D53" s="14" t="inlineStr">
         <is>
           <t>한화시스템</t>
         </is>
       </c>
-      <c r="F50" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="15" t="n">
+      <c r="E53" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F53" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="12" t="n">
         <v>45772</v>
       </c>
-      <c r="B51" s="15" t="n">
+      <c r="B54" s="12" t="n">
         <v>45868</v>
       </c>
-      <c r="C51" s="16" t="inlineStr">
+      <c r="C54" s="13" t="inlineStr">
         <is>
           <t>009830</t>
         </is>
       </c>
-      <c r="D51" s="17" t="inlineStr">
+      <c r="D54" s="14" t="inlineStr">
         <is>
           <t>한화솔루션</t>
         </is>
       </c>
-      <c r="F51" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="15" t="n">
+      <c r="E54" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F54" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="12" t="n">
         <v>45868</v>
       </c>
-      <c r="B52" s="15" t="n">
+      <c r="B55" s="12" t="n">
         <v>45868</v>
       </c>
-      <c r="C52" s="16" t="inlineStr">
+      <c r="C55" s="13" t="inlineStr">
         <is>
           <t>009150</t>
         </is>
       </c>
-      <c r="D52" s="17" t="inlineStr">
+      <c r="D55" s="14" t="inlineStr">
         <is>
           <t>삼성전기</t>
         </is>
       </c>
-      <c r="F52" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="15" t="n">
+      <c r="E55" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F55" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="12" t="n">
         <v>45867</v>
       </c>
-      <c r="B53" s="15" t="n">
+      <c r="B56" s="12" t="n">
         <v>45867</v>
       </c>
-      <c r="C53" s="16" t="inlineStr">
+      <c r="C56" s="13" t="inlineStr">
         <is>
           <t>489790</t>
         </is>
       </c>
-      <c r="D53" s="17" t="inlineStr">
+      <c r="D56" s="14" t="inlineStr">
         <is>
           <t>한화비전</t>
         </is>
       </c>
-      <c r="F53" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="15" t="n">
+      <c r="E56" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F56" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="12" t="n">
         <v>45862</v>
       </c>
-      <c r="B54" s="15" t="n">
+      <c r="B57" s="12" t="n">
         <v>45867</v>
       </c>
-      <c r="C54" s="16" t="inlineStr">
+      <c r="C57" s="13" t="inlineStr">
         <is>
           <t>042670</t>
         </is>
       </c>
-      <c r="D54" s="17" t="inlineStr">
+      <c r="D57" s="14" t="inlineStr">
         <is>
           <t>HD현대인프라코어</t>
         </is>
       </c>
-      <c r="F54" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="15" t="n">
+      <c r="E57" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F57" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="12" t="n">
         <v>45861</v>
       </c>
-      <c r="B55" s="15" t="n">
+      <c r="B58" s="12" t="n">
         <v>45861</v>
       </c>
-      <c r="C55" s="16" t="inlineStr">
+      <c r="C58" s="13" t="inlineStr">
         <is>
           <t>484120</t>
         </is>
       </c>
-      <c r="D55" s="17" t="inlineStr">
+      <c r="D58" s="14" t="inlineStr">
         <is>
           <t>도우인시스</t>
         </is>
       </c>
-      <c r="F55" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="15" t="n">
+      <c r="E58" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F58" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="12" t="n">
         <v>45846</v>
       </c>
-      <c r="B56" s="15" t="n">
+      <c r="B59" s="12" t="n">
         <v>45861</v>
       </c>
-      <c r="C56" s="16" t="inlineStr">
+      <c r="C59" s="13" t="inlineStr">
         <is>
           <t>008970</t>
         </is>
       </c>
-      <c r="D56" s="17" t="inlineStr">
+      <c r="D59" s="14" t="inlineStr">
         <is>
           <t>KBI동양철관</t>
         </is>
       </c>
-      <c r="F56" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="15" t="n">
+      <c r="E59" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F59" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="12" t="n">
         <v>45860</v>
       </c>
-      <c r="B57" s="15" t="n">
+      <c r="B60" s="12" t="n">
         <v>45860</v>
       </c>
-      <c r="C57" s="16" t="inlineStr">
+      <c r="C60" s="13" t="inlineStr">
         <is>
           <t>037270</t>
         </is>
       </c>
-      <c r="D57" s="17" t="inlineStr">
+      <c r="D60" s="14" t="inlineStr">
         <is>
           <t>YG PLUS</t>
         </is>
       </c>
-      <c r="F57" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="15" t="n">
+      <c r="E60" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F60" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="12" t="n">
         <v>45856</v>
       </c>
-      <c r="B58" s="15" t="n">
+      <c r="B61" s="12" t="n">
         <v>45856</v>
       </c>
-      <c r="C58" s="16" t="inlineStr">
+      <c r="C61" s="13" t="inlineStr">
         <is>
           <t>003670</t>
         </is>
       </c>
-      <c r="D58" s="17" t="inlineStr">
+      <c r="D61" s="14" t="inlineStr">
         <is>
           <t>포스코퓨처엠</t>
         </is>
       </c>
-      <c r="F58" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="15" t="n">
+      <c r="E61" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F61" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="12" t="n">
         <v>45856</v>
       </c>
-      <c r="B59" s="15" t="n">
+      <c r="B62" s="12" t="n">
         <v>45856</v>
       </c>
-      <c r="C59" s="16" t="inlineStr">
+      <c r="C62" s="13" t="inlineStr">
         <is>
           <t>141080</t>
         </is>
       </c>
-      <c r="D59" s="17" t="inlineStr">
+      <c r="D62" s="14" t="inlineStr">
         <is>
           <t>리가켐바이오</t>
         </is>
       </c>
-      <c r="F59" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="15" t="n">
+      <c r="E62" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F62" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="12" t="n">
         <v>45854</v>
       </c>
-      <c r="B60" s="15" t="n">
+      <c r="B63" s="12" t="n">
         <v>45854</v>
       </c>
-      <c r="C60" s="16" t="inlineStr">
+      <c r="C63" s="13" t="inlineStr">
         <is>
           <t>294570</t>
         </is>
       </c>
-      <c r="D60" s="17" t="inlineStr">
+      <c r="D63" s="14" t="inlineStr">
         <is>
           <t>쿠콘</t>
         </is>
       </c>
-      <c r="F60" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="15" t="n">
+      <c r="E63" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F63" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="12" t="n">
         <v>45854</v>
       </c>
-      <c r="B61" s="15" t="n">
+      <c r="B64" s="12" t="n">
         <v>45854</v>
       </c>
-      <c r="C61" s="16" t="inlineStr">
+      <c r="C64" s="13" t="inlineStr">
         <is>
           <t>441270</t>
         </is>
       </c>
-      <c r="D61" s="17" t="inlineStr">
+      <c r="D64" s="14" t="inlineStr">
         <is>
           <t>파인엠텍</t>
         </is>
       </c>
-      <c r="F61" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="15" t="n">
+      <c r="E64" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F64" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="12" t="n">
         <v>45849</v>
       </c>
-      <c r="B62" s="15" t="n">
+      <c r="B65" s="12" t="n">
         <v>45849</v>
       </c>
-      <c r="C62" s="16" t="inlineStr">
+      <c r="C65" s="13" t="inlineStr">
         <is>
           <t>402340</t>
         </is>
       </c>
-      <c r="D62" s="17" t="inlineStr">
+      <c r="D65" s="14" t="inlineStr">
         <is>
           <t>SK스퀘어</t>
         </is>
       </c>
-      <c r="F62" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="15" t="n">
+      <c r="E65" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F65" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="12" t="n">
         <v>45841</v>
       </c>
-      <c r="B63" s="15" t="n">
+      <c r="B66" s="12" t="n">
         <v>45842</v>
       </c>
-      <c r="C63" s="16" t="inlineStr">
+      <c r="C66" s="13" t="inlineStr">
         <is>
           <t>005490</t>
         </is>
       </c>
-      <c r="D63" s="17" t="inlineStr">
+      <c r="D66" s="14" t="inlineStr">
         <is>
           <t>POSCO홀딩스</t>
         </is>
       </c>
-      <c r="F63" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="15" t="n">
+      <c r="E66" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F66" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="12" t="n">
         <v>45840</v>
       </c>
-      <c r="B64" s="15" t="n">
+      <c r="B67" s="12" t="n">
         <v>45840</v>
       </c>
-      <c r="C64" s="16" t="inlineStr">
+      <c r="C67" s="13" t="inlineStr">
         <is>
           <t>267270</t>
         </is>
       </c>
-      <c r="D64" s="17" t="inlineStr">
+      <c r="D67" s="14" t="inlineStr">
         <is>
           <t>HD현대건설기계</t>
         </is>
       </c>
-      <c r="F64" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="15" t="n">
+      <c r="E67" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F67" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="12" t="n">
         <v>45839</v>
       </c>
-      <c r="B65" s="15" t="n">
+      <c r="B68" s="12" t="n">
         <v>45839</v>
       </c>
-      <c r="C65" s="16" t="inlineStr">
+      <c r="C68" s="13" t="inlineStr">
         <is>
           <t>000880</t>
         </is>
       </c>
-      <c r="D65" s="17" t="inlineStr">
+      <c r="D68" s="14" t="inlineStr">
         <is>
           <t>한화</t>
         </is>
       </c>
-      <c r="F65" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="15" t="n">
+      <c r="E68" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F68" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="12" t="n">
         <v>43997</v>
       </c>
-      <c r="B66" s="15" t="n">
+      <c r="B69" s="12" t="n">
         <v>45839</v>
       </c>
-      <c r="C66" s="16" t="inlineStr">
+      <c r="C69" s="13" t="inlineStr">
         <is>
           <t>034730</t>
         </is>
       </c>
-      <c r="D66" s="17" t="inlineStr">
+      <c r="D69" s="14" t="inlineStr">
         <is>
           <t>SK</t>
         </is>
       </c>
-      <c r="F66" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="15" t="n">
+      <c r="E69" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F69" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="12" t="n">
         <v>45838</v>
       </c>
-      <c r="B67" s="15" t="n">
+      <c r="B70" s="12" t="n">
         <v>45839</v>
       </c>
-      <c r="C67" s="16" t="inlineStr">
+      <c r="C70" s="13" t="inlineStr">
         <is>
           <t>096770</t>
         </is>
       </c>
-      <c r="D67" s="17" t="inlineStr">
+      <c r="D70" s="14" t="inlineStr">
         <is>
           <t>SK이노베이션</t>
         </is>
       </c>
-      <c r="F67" s="19" t="n">
+      <c r="E70" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F70" s="16" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: push latest changes
</commit_message>
<xml_diff>
--- a/output/turnover_universe.xlsx
+++ b/output/turnover_universe.xlsx
@@ -573,7 +573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H74"/>
+  <dimension ref="A1:H80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -617,7 +617,7 @@
       </c>
       <c r="H1" s="13" t="inlineStr">
         <is>
-          <t>최종 업데이트: 2025-10-22</t>
+          <t>최종 업데이트: 2025-10-29</t>
         </is>
       </c>
     </row>
@@ -626,7 +626,7 @@
         <v>45942</v>
       </c>
       <c r="B2" s="14" t="n">
-        <v>45952</v>
+        <v>45959</v>
       </c>
       <c r="C2" s="15" t="inlineStr">
         <is>
@@ -639,10 +639,10 @@
         </is>
       </c>
       <c r="E2" s="17" t="n">
-        <v>24644.13</v>
+        <v>34789.85</v>
       </c>
       <c r="F2" s="18" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3">
@@ -650,7 +650,7 @@
         <v>45942</v>
       </c>
       <c r="B3" s="14" t="n">
-        <v>45952</v>
+        <v>45959</v>
       </c>
       <c r="C3" s="15" t="inlineStr">
         <is>
@@ -663,10 +663,10 @@
         </is>
       </c>
       <c r="E3" s="17" t="n">
-        <v>26196.57</v>
+        <v>52358.47</v>
       </c>
       <c r="F3" s="18" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4">
@@ -674,7 +674,7 @@
         <v>45942</v>
       </c>
       <c r="B4" s="14" t="n">
-        <v>45952</v>
+        <v>45959</v>
       </c>
       <c r="C4" s="15" t="inlineStr">
         <is>
@@ -687,34 +687,34 @@
         </is>
       </c>
       <c r="E4" s="17" t="n">
-        <v>8626.440000000001</v>
+        <v>39513.58</v>
       </c>
       <c r="F4" s="18" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
-        <v>45942</v>
+        <v>45604</v>
       </c>
       <c r="B5" s="14" t="n">
-        <v>45951</v>
+        <v>45959</v>
       </c>
       <c r="C5" s="15" t="inlineStr">
         <is>
-          <t>035420</t>
+          <t>042660</t>
         </is>
       </c>
       <c r="D5" s="16" t="inlineStr">
         <is>
-          <t>NAVER</t>
+          <t>한화오션</t>
         </is>
       </c>
       <c r="E5" s="17" t="n">
-        <v>5807.59</v>
+        <v>15944.28</v>
       </c>
       <c r="F5" s="18" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6">
@@ -722,71 +722,71 @@
         <v>45942</v>
       </c>
       <c r="B6" s="14" t="n">
-        <v>45951</v>
+        <v>45959</v>
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>042700</t>
+          <t>035420</t>
         </is>
       </c>
       <c r="D6" s="16" t="inlineStr">
         <is>
-          <t>한미반도체</t>
+          <t>NAVER</t>
         </is>
       </c>
       <c r="E6" s="17" t="n">
-        <v>9017.120000000001</v>
+        <v>12265.68</v>
       </c>
       <c r="F6" s="18" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>45947</v>
+        <v>45730</v>
       </c>
       <c r="B7" s="14" t="n">
-        <v>45952</v>
+        <v>45959</v>
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>086520</t>
+          <t>006400</t>
         </is>
       </c>
       <c r="D7" s="16" t="inlineStr">
         <is>
-          <t>에코프로</t>
+          <t>삼성SDI</t>
         </is>
       </c>
       <c r="E7" s="17" t="n">
-        <v>16325.35</v>
+        <v>13351.78</v>
       </c>
       <c r="F7" s="18" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>45604</v>
+        <v>45942</v>
       </c>
       <c r="B8" s="14" t="n">
-        <v>45952</v>
+        <v>45959</v>
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>042660</t>
+          <t>042700</t>
         </is>
       </c>
       <c r="D8" s="16" t="inlineStr">
         <is>
-          <t>한화오션</t>
+          <t>한미반도체</t>
         </is>
       </c>
       <c r="E8" s="17" t="n">
-        <v>18406.15</v>
+        <v>9485.610000000001</v>
       </c>
       <c r="F8" s="18" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9">
@@ -794,7 +794,7 @@
         <v>45833</v>
       </c>
       <c r="B9" s="14" t="n">
-        <v>45952</v>
+        <v>45959</v>
       </c>
       <c r="C9" s="15" t="inlineStr">
         <is>
@@ -807,151 +807,151 @@
         </is>
       </c>
       <c r="E9" s="17" t="n">
-        <v>5049</v>
+        <v>12484.9</v>
       </c>
       <c r="F9" s="18" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>45874</v>
+        <v>45947</v>
       </c>
       <c r="B10" s="14" t="n">
-        <v>45949</v>
+        <v>45958</v>
       </c>
       <c r="C10" s="15" t="inlineStr">
         <is>
-          <t>247540</t>
+          <t>086520</t>
         </is>
       </c>
       <c r="D10" s="16" t="inlineStr">
         <is>
-          <t>에코프로비엠</t>
+          <t>에코프로</t>
         </is>
       </c>
       <c r="E10" s="17" t="n">
-        <v>16882.57</v>
+        <v>8493.91</v>
       </c>
       <c r="F10" s="18" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>45730</v>
+        <v>45856</v>
       </c>
       <c r="B11" s="14" t="n">
-        <v>45949</v>
+        <v>45958</v>
       </c>
       <c r="C11" s="15" t="inlineStr">
         <is>
-          <t>006400</t>
+          <t>003670</t>
         </is>
       </c>
       <c r="D11" s="16" t="inlineStr">
         <is>
-          <t>삼성SDI</t>
+          <t>포스코퓨처엠</t>
         </is>
       </c>
       <c r="E11" s="17" t="n">
-        <v>11005.97</v>
+        <v>5493.64</v>
       </c>
       <c r="F11" s="18" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>45947</v>
+        <v>45874</v>
       </c>
       <c r="B12" s="14" t="n">
-        <v>45952</v>
+        <v>45957</v>
       </c>
       <c r="C12" s="15" t="inlineStr">
         <is>
-          <t>051910</t>
+          <t>247540</t>
         </is>
       </c>
       <c r="D12" s="16" t="inlineStr">
         <is>
-          <t>LG화학</t>
+          <t>에코프로비엠</t>
         </is>
       </c>
       <c r="E12" s="17" t="n">
-        <v>9404.630000000001</v>
+        <v>12071.61</v>
       </c>
       <c r="F12" s="18" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>45947</v>
+        <v>45365</v>
       </c>
       <c r="B13" s="14" t="n">
-        <v>45949</v>
+        <v>45959</v>
       </c>
       <c r="C13" s="15" t="inlineStr">
         <is>
-          <t>450080</t>
+          <t>010140</t>
         </is>
       </c>
       <c r="D13" s="16" t="inlineStr">
         <is>
-          <t>에코프로머티</t>
+          <t>삼성중공업</t>
         </is>
       </c>
       <c r="E13" s="17" t="n">
-        <v>7222.29</v>
+        <v>9568.76</v>
       </c>
       <c r="F13" s="18" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>45946</v>
+        <v>44876</v>
       </c>
       <c r="B14" s="14" t="n">
-        <v>45949</v>
+        <v>45959</v>
       </c>
       <c r="C14" s="15" t="inlineStr">
         <is>
-          <t>373220</t>
+          <t>035720</t>
         </is>
       </c>
       <c r="D14" s="16" t="inlineStr">
         <is>
-          <t>LG에너지솔루션</t>
+          <t>카카오</t>
         </is>
       </c>
       <c r="E14" s="17" t="n">
-        <v>6561.16</v>
+        <v>16671.6</v>
       </c>
       <c r="F14" s="18" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>45853</v>
+        <v>45947</v>
       </c>
       <c r="B15" s="14" t="n">
-        <v>45949</v>
+        <v>45952</v>
       </c>
       <c r="C15" s="15" t="inlineStr">
         <is>
-          <t>015760</t>
+          <t>051910</t>
         </is>
       </c>
       <c r="D15" s="16" t="inlineStr">
         <is>
-          <t>한국전력</t>
+          <t>LG화학</t>
         </is>
       </c>
       <c r="E15" s="17" t="n">
-        <v>6619.35</v>
+        <v>9404.630000000001</v>
       </c>
       <c r="F15" s="18" t="n">
         <v>3</v>
@@ -959,23 +959,23 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>45856</v>
+        <v>45947</v>
       </c>
       <c r="B16" s="14" t="n">
         <v>45949</v>
       </c>
       <c r="C16" s="15" t="inlineStr">
         <is>
-          <t>003670</t>
+          <t>450080</t>
         </is>
       </c>
       <c r="D16" s="16" t="inlineStr">
         <is>
-          <t>포스코퓨처엠</t>
+          <t>에코프로머티</t>
         </is>
       </c>
       <c r="E16" s="17" t="n">
-        <v>5770.900000000001</v>
+        <v>7222.29</v>
       </c>
       <c r="F16" s="18" t="n">
         <v>3</v>
@@ -983,71 +983,71 @@
     </row>
     <row r="17">
       <c r="A17" s="14" t="n">
-        <v>45694</v>
+        <v>45946</v>
       </c>
       <c r="B17" s="14" t="n">
-        <v>45952</v>
+        <v>45949</v>
       </c>
       <c r="C17" s="15" t="inlineStr">
         <is>
-          <t>064350</t>
+          <t>373220</t>
         </is>
       </c>
       <c r="D17" s="16" t="inlineStr">
         <is>
-          <t>현대로템</t>
+          <t>LG에너지솔루션</t>
         </is>
       </c>
       <c r="E17" s="17" t="n">
-        <v>6133.97</v>
+        <v>6561.16</v>
       </c>
       <c r="F17" s="18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="14" t="n">
-        <v>44876</v>
+        <v>45853</v>
       </c>
       <c r="B18" s="14" t="n">
-        <v>45951</v>
+        <v>45949</v>
       </c>
       <c r="C18" s="15" t="inlineStr">
         <is>
-          <t>035720</t>
+          <t>015760</t>
         </is>
       </c>
       <c r="D18" s="16" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>한국전력</t>
         </is>
       </c>
       <c r="E18" s="17" t="n">
-        <v>8538.540000000001</v>
+        <v>6619.35</v>
       </c>
       <c r="F18" s="18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="14" t="n">
-        <v>45947</v>
+        <v>45958</v>
       </c>
       <c r="B19" s="14" t="n">
-        <v>45949</v>
+        <v>45959</v>
       </c>
       <c r="C19" s="15" t="inlineStr">
         <is>
-          <t>066970</t>
+          <t>336260</t>
         </is>
       </c>
       <c r="D19" s="16" t="inlineStr">
         <is>
-          <t>엘앤에프</t>
+          <t>두산퓨얼셀</t>
         </is>
       </c>
       <c r="E19" s="17" t="n">
-        <v>5810.01</v>
+        <v>5907.51</v>
       </c>
       <c r="F19" s="18" t="n">
         <v>2</v>
@@ -1055,23 +1055,23 @@
     </row>
     <row r="20">
       <c r="A20" s="14" t="n">
-        <v>45947</v>
+        <v>45957</v>
       </c>
       <c r="B20" s="14" t="n">
-        <v>45949</v>
+        <v>45959</v>
       </c>
       <c r="C20" s="15" t="inlineStr">
         <is>
-          <t>000150</t>
+          <t>000720</t>
         </is>
       </c>
       <c r="D20" s="16" t="inlineStr">
         <is>
-          <t>두산</t>
+          <t>현대건설</t>
         </is>
       </c>
       <c r="E20" s="17" t="n">
-        <v>5742.17</v>
+        <v>7859.2</v>
       </c>
       <c r="F20" s="18" t="n">
         <v>2</v>
@@ -1079,23 +1079,23 @@
     </row>
     <row r="21">
       <c r="A21" s="14" t="n">
-        <v>45916</v>
+        <v>45650</v>
       </c>
       <c r="B21" s="14" t="n">
-        <v>45945</v>
+        <v>45957</v>
       </c>
       <c r="C21" s="15" t="inlineStr">
         <is>
-          <t>125490</t>
+          <t>196170</t>
         </is>
       </c>
       <c r="D21" s="16" t="inlineStr">
         <is>
-          <t>한라캐스트</t>
+          <t>알테오젠</t>
         </is>
       </c>
       <c r="E21" s="17" t="n">
-        <v>5614.12</v>
+        <v>6894.2</v>
       </c>
       <c r="F21" s="18" t="n">
         <v>2</v>
@@ -1103,143 +1103,143 @@
     </row>
     <row r="22">
       <c r="A22" s="14" t="n">
-        <v>45951</v>
+        <v>45876</v>
       </c>
       <c r="B22" s="14" t="n">
-        <v>45951</v>
+        <v>45957</v>
       </c>
       <c r="C22" s="15" t="inlineStr">
         <is>
-          <t>090710</t>
+          <t>097230</t>
         </is>
       </c>
       <c r="D22" s="16" t="inlineStr">
         <is>
-          <t>휴림로봇</t>
+          <t>HJ중공업</t>
         </is>
       </c>
       <c r="E22" s="17" t="n">
-        <v>7343.57</v>
+        <v>6016.41</v>
       </c>
       <c r="F22" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="14" t="n">
-        <v>45943</v>
+        <v>45694</v>
       </c>
       <c r="B23" s="14" t="n">
-        <v>45943</v>
+        <v>45952</v>
       </c>
       <c r="C23" s="15" t="inlineStr">
         <is>
-          <t>466100</t>
+          <t>064350</t>
         </is>
       </c>
       <c r="D23" s="16" t="inlineStr">
         <is>
-          <t>클로봇</t>
+          <t>현대로템</t>
         </is>
       </c>
       <c r="E23" s="17" t="n">
-        <v>6494.860000000001</v>
+        <v>6133.97</v>
       </c>
       <c r="F23" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="14" t="n">
-        <v>45942</v>
+        <v>45947</v>
       </c>
       <c r="B24" s="14" t="n">
-        <v>45942</v>
+        <v>45949</v>
       </c>
       <c r="C24" s="15" t="inlineStr">
         <is>
-          <t>108490</t>
+          <t>066970</t>
         </is>
       </c>
       <c r="D24" s="16" t="inlineStr">
         <is>
-          <t>로보티즈</t>
+          <t>엘앤에프</t>
         </is>
       </c>
       <c r="E24" s="17" t="n">
-        <v>8159.77</v>
+        <v>5810.01</v>
       </c>
       <c r="F24" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="14" t="n">
-        <v>45942</v>
+        <v>45947</v>
       </c>
       <c r="B25" s="14" t="n">
-        <v>45942</v>
+        <v>45949</v>
       </c>
       <c r="C25" s="15" t="inlineStr">
         <is>
-          <t>005935</t>
+          <t>000150</t>
         </is>
       </c>
       <c r="D25" s="16" t="inlineStr">
         <is>
-          <t>삼성전자우</t>
+          <t>두산</t>
         </is>
       </c>
       <c r="E25" s="17" t="n">
-        <v>5438.03</v>
+        <v>5742.17</v>
       </c>
       <c r="F25" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="14" t="n">
-        <v>44512</v>
+        <v>45916</v>
       </c>
       <c r="B26" s="14" t="n">
-        <v>45929</v>
+        <v>45945</v>
       </c>
       <c r="C26" s="15" t="inlineStr">
         <is>
-          <t>249420</t>
+          <t>125490</t>
         </is>
       </c>
       <c r="D26" s="16" t="inlineStr">
         <is>
-          <t>일동제약</t>
+          <t>한라캐스트</t>
         </is>
       </c>
       <c r="E26" s="17" t="n">
-        <v>9183</v>
+        <v>5614.12</v>
       </c>
       <c r="F26" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="14" t="n">
-        <v>45849</v>
+        <v>45959</v>
       </c>
       <c r="B27" s="14" t="n">
-        <v>45929</v>
+        <v>45959</v>
       </c>
       <c r="C27" s="15" t="inlineStr">
         <is>
-          <t>041190</t>
+          <t>001440</t>
         </is>
       </c>
       <c r="D27" s="16" t="inlineStr">
         <is>
-          <t>우리기술투자</t>
+          <t>대한전선</t>
         </is>
       </c>
       <c r="E27" s="17" t="n">
-        <v>5517</v>
+        <v>5087.57</v>
       </c>
       <c r="F27" s="18" t="n">
         <v>1</v>
@@ -1247,23 +1247,23 @@
     </row>
     <row r="28">
       <c r="A28" s="14" t="n">
-        <v>45849</v>
+        <v>45958</v>
       </c>
       <c r="B28" s="14" t="n">
-        <v>45926</v>
+        <v>45958</v>
       </c>
       <c r="C28" s="15" t="inlineStr">
         <is>
-          <t>060250</t>
+          <t>011790</t>
         </is>
       </c>
       <c r="D28" s="16" t="inlineStr">
         <is>
-          <t>NHN KCP</t>
+          <t>SKC</t>
         </is>
       </c>
       <c r="E28" s="17" t="n">
-        <v>9171</v>
+        <v>5001.6</v>
       </c>
       <c r="F28" s="18" t="n">
         <v>1</v>
@@ -1271,23 +1271,23 @@
     </row>
     <row r="29">
       <c r="A29" s="14" t="n">
-        <v>45925</v>
+        <v>45957</v>
       </c>
       <c r="B29" s="14" t="n">
-        <v>45925</v>
+        <v>45957</v>
       </c>
       <c r="C29" s="15" t="inlineStr">
         <is>
-          <t>277810</t>
+          <t>128940</t>
         </is>
       </c>
       <c r="D29" s="16" t="inlineStr">
         <is>
-          <t>레인보우로보틱스</t>
+          <t>한미약품</t>
         </is>
       </c>
       <c r="E29" s="17" t="n">
-        <v>7211</v>
+        <v>7324.5</v>
       </c>
       <c r="F29" s="18" t="n">
         <v>1</v>
@@ -1295,23 +1295,23 @@
     </row>
     <row r="30">
       <c r="A30" s="14" t="n">
-        <v>45650</v>
+        <v>45957</v>
       </c>
       <c r="B30" s="14" t="n">
-        <v>45924</v>
+        <v>45957</v>
       </c>
       <c r="C30" s="15" t="inlineStr">
         <is>
-          <t>196170</t>
+          <t>352820</t>
         </is>
       </c>
       <c r="D30" s="16" t="inlineStr">
         <is>
-          <t>알테오젠</t>
+          <t>하이브</t>
         </is>
       </c>
       <c r="E30" s="17" t="n">
-        <v>5188</v>
+        <v>5473.690000000001</v>
       </c>
       <c r="F30" s="18" t="n">
         <v>1</v>
@@ -1319,23 +1319,23 @@
     </row>
     <row r="31">
       <c r="A31" s="14" t="n">
-        <v>44515</v>
+        <v>45951</v>
       </c>
       <c r="B31" s="14" t="n">
-        <v>45923</v>
+        <v>45951</v>
       </c>
       <c r="C31" s="15" t="inlineStr">
         <is>
-          <t>068270</t>
+          <t>090710</t>
         </is>
       </c>
       <c r="D31" s="16" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>휴림로봇</t>
         </is>
       </c>
       <c r="E31" s="17" t="n">
-        <v>5000</v>
+        <v>7343.57</v>
       </c>
       <c r="F31" s="18" t="n">
         <v>1</v>
@@ -1343,23 +1343,23 @@
     </row>
     <row r="32">
       <c r="A32" s="14" t="n">
-        <v>45922</v>
+        <v>45943</v>
       </c>
       <c r="B32" s="14" t="n">
-        <v>45923</v>
+        <v>45943</v>
       </c>
       <c r="C32" s="15" t="inlineStr">
         <is>
-          <t>347850</t>
+          <t>466100</t>
         </is>
       </c>
       <c r="D32" s="16" t="inlineStr">
         <is>
-          <t>디앤디파마텍</t>
+          <t>클로봇</t>
         </is>
       </c>
       <c r="E32" s="17" t="n">
-        <v>5000</v>
+        <v>6494.860000000001</v>
       </c>
       <c r="F32" s="18" t="n">
         <v>1</v>
@@ -1367,23 +1367,23 @@
     </row>
     <row r="33">
       <c r="A33" s="14" t="n">
-        <v>45377</v>
+        <v>45942</v>
       </c>
       <c r="B33" s="14" t="n">
-        <v>45919</v>
+        <v>45942</v>
       </c>
       <c r="C33" s="15" t="inlineStr">
         <is>
-          <t>000250</t>
+          <t>108490</t>
         </is>
       </c>
       <c r="D33" s="16" t="inlineStr">
         <is>
-          <t>삼천당제약</t>
+          <t>로보티즈</t>
         </is>
       </c>
       <c r="E33" s="17" t="n">
-        <v>5000</v>
+        <v>8159.77</v>
       </c>
       <c r="F33" s="18" t="n">
         <v>1</v>
@@ -1391,23 +1391,23 @@
     </row>
     <row r="34">
       <c r="A34" s="14" t="n">
-        <v>45839</v>
+        <v>45942</v>
       </c>
       <c r="B34" s="14" t="n">
-        <v>45919</v>
+        <v>45942</v>
       </c>
       <c r="C34" s="15" t="inlineStr">
         <is>
-          <t>064260</t>
+          <t>005935</t>
         </is>
       </c>
       <c r="D34" s="16" t="inlineStr">
         <is>
-          <t>다날</t>
+          <t>삼성전자우</t>
         </is>
       </c>
       <c r="E34" s="17" t="n">
-        <v>5000</v>
+        <v>5438.03</v>
       </c>
       <c r="F34" s="18" t="n">
         <v>1</v>
@@ -1415,23 +1415,23 @@
     </row>
     <row r="35">
       <c r="A35" s="14" t="n">
-        <v>45918</v>
+        <v>44512</v>
       </c>
       <c r="B35" s="14" t="n">
-        <v>45919</v>
+        <v>45929</v>
       </c>
       <c r="C35" s="15" t="inlineStr">
         <is>
-          <t>090360</t>
+          <t>249420</t>
         </is>
       </c>
       <c r="D35" s="16" t="inlineStr">
         <is>
-          <t>로보스타</t>
+          <t>일동제약</t>
         </is>
       </c>
       <c r="E35" s="17" t="n">
-        <v>5000</v>
+        <v>9183</v>
       </c>
       <c r="F35" s="18" t="n">
         <v>1</v>
@@ -1439,23 +1439,23 @@
     </row>
     <row r="36">
       <c r="A36" s="14" t="n">
-        <v>45708</v>
+        <v>45849</v>
       </c>
       <c r="B36" s="14" t="n">
-        <v>45919</v>
+        <v>45929</v>
       </c>
       <c r="C36" s="15" t="inlineStr">
         <is>
-          <t>047810</t>
+          <t>041190</t>
         </is>
       </c>
       <c r="D36" s="16" t="inlineStr">
         <is>
-          <t>한국항공우주</t>
+          <t>우리기술투자</t>
         </is>
       </c>
       <c r="E36" s="17" t="n">
-        <v>5000</v>
+        <v>5517</v>
       </c>
       <c r="F36" s="18" t="n">
         <v>1</v>
@@ -1463,23 +1463,23 @@
     </row>
     <row r="37">
       <c r="A37" s="14" t="n">
-        <v>45883</v>
+        <v>45849</v>
       </c>
       <c r="B37" s="14" t="n">
-        <v>45912</v>
+        <v>45926</v>
       </c>
       <c r="C37" s="15" t="inlineStr">
         <is>
-          <t>456160</t>
+          <t>060250</t>
         </is>
       </c>
       <c r="D37" s="16" t="inlineStr">
         <is>
-          <t>지투지바이오</t>
+          <t>NHN KCP</t>
         </is>
       </c>
       <c r="E37" s="17" t="n">
-        <v>5000</v>
+        <v>9171</v>
       </c>
       <c r="F37" s="18" t="n">
         <v>1</v>
@@ -1487,23 +1487,23 @@
     </row>
     <row r="38">
       <c r="A38" s="14" t="n">
-        <v>45912</v>
+        <v>45925</v>
       </c>
       <c r="B38" s="14" t="n">
-        <v>45912</v>
+        <v>45925</v>
       </c>
       <c r="C38" s="15" t="inlineStr">
         <is>
-          <t>004370</t>
+          <t>277810</t>
         </is>
       </c>
       <c r="D38" s="16" t="inlineStr">
         <is>
-          <t>농심</t>
+          <t>레인보우로보틱스</t>
         </is>
       </c>
       <c r="E38" s="17" t="n">
-        <v>5000</v>
+        <v>7211</v>
       </c>
       <c r="F38" s="18" t="n">
         <v>1</v>
@@ -1511,19 +1511,19 @@
     </row>
     <row r="39">
       <c r="A39" s="14" t="n">
-        <v>45911</v>
+        <v>44515</v>
       </c>
       <c r="B39" s="14" t="n">
-        <v>45912</v>
+        <v>45923</v>
       </c>
       <c r="C39" s="15" t="inlineStr">
         <is>
-          <t>100090</t>
+          <t>068270</t>
         </is>
       </c>
       <c r="D39" s="16" t="inlineStr">
         <is>
-          <t>SK오션플랜트</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="E39" s="17" t="n">
@@ -1535,19 +1535,19 @@
     </row>
     <row r="40">
       <c r="A40" s="14" t="n">
-        <v>45876</v>
+        <v>45922</v>
       </c>
       <c r="B40" s="14" t="n">
-        <v>45910</v>
+        <v>45923</v>
       </c>
       <c r="C40" s="15" t="inlineStr">
         <is>
-          <t>097230</t>
+          <t>347850</t>
         </is>
       </c>
       <c r="D40" s="16" t="inlineStr">
         <is>
-          <t>HJ중공업</t>
+          <t>디앤디파마텍</t>
         </is>
       </c>
       <c r="E40" s="17" t="n">
@@ -1559,19 +1559,19 @@
     </row>
     <row r="41">
       <c r="A41" s="14" t="n">
-        <v>45908</v>
+        <v>45377</v>
       </c>
       <c r="B41" s="14" t="n">
-        <v>45910</v>
+        <v>45919</v>
       </c>
       <c r="C41" s="15" t="inlineStr">
         <is>
-          <t>075580</t>
+          <t>000250</t>
         </is>
       </c>
       <c r="D41" s="16" t="inlineStr">
         <is>
-          <t>세진중공업</t>
+          <t>삼천당제약</t>
         </is>
       </c>
       <c r="E41" s="17" t="n">
@@ -1583,19 +1583,19 @@
     </row>
     <row r="42">
       <c r="A42" s="14" t="n">
-        <v>45908</v>
+        <v>45839</v>
       </c>
       <c r="B42" s="14" t="n">
-        <v>45908</v>
+        <v>45919</v>
       </c>
       <c r="C42" s="15" t="inlineStr">
         <is>
-          <t>290650</t>
+          <t>064260</t>
         </is>
       </c>
       <c r="D42" s="16" t="inlineStr">
         <is>
-          <t>엘앤씨바이오</t>
+          <t>다날</t>
         </is>
       </c>
       <c r="E42" s="17" t="n">
@@ -1607,19 +1607,19 @@
     </row>
     <row r="43">
       <c r="A43" s="14" t="n">
-        <v>45898</v>
+        <v>45918</v>
       </c>
       <c r="B43" s="14" t="n">
-        <v>45898</v>
+        <v>45919</v>
       </c>
       <c r="C43" s="15" t="inlineStr">
         <is>
-          <t>082740</t>
+          <t>090360</t>
         </is>
       </c>
       <c r="D43" s="16" t="inlineStr">
         <is>
-          <t>한화엔진</t>
+          <t>로보스타</t>
         </is>
       </c>
       <c r="E43" s="17" t="n">
@@ -1631,19 +1631,19 @@
     </row>
     <row r="44">
       <c r="A44" s="14" t="n">
-        <v>45897</v>
+        <v>45708</v>
       </c>
       <c r="B44" s="14" t="n">
-        <v>45897</v>
+        <v>45919</v>
       </c>
       <c r="C44" s="15" t="inlineStr">
         <is>
-          <t>460930</t>
+          <t>047810</t>
         </is>
       </c>
       <c r="D44" s="16" t="inlineStr">
         <is>
-          <t>현대힘스</t>
+          <t>한국항공우주</t>
         </is>
       </c>
       <c r="E44" s="17" t="n">
@@ -1655,19 +1655,19 @@
     </row>
     <row r="45">
       <c r="A45" s="14" t="n">
-        <v>45897</v>
+        <v>45883</v>
       </c>
       <c r="B45" s="14" t="n">
-        <v>45897</v>
+        <v>45912</v>
       </c>
       <c r="C45" s="15" t="inlineStr">
         <is>
-          <t>009540</t>
+          <t>456160</t>
         </is>
       </c>
       <c r="D45" s="16" t="inlineStr">
         <is>
-          <t>HD한국조선해양</t>
+          <t>지투지바이오</t>
         </is>
       </c>
       <c r="E45" s="17" t="n">
@@ -1679,19 +1679,19 @@
     </row>
     <row r="46">
       <c r="A46" s="14" t="n">
-        <v>45896</v>
+        <v>45912</v>
       </c>
       <c r="B46" s="14" t="n">
-        <v>45897</v>
+        <v>45912</v>
       </c>
       <c r="C46" s="15" t="inlineStr">
         <is>
-          <t>010620</t>
+          <t>004370</t>
         </is>
       </c>
       <c r="D46" s="16" t="inlineStr">
         <is>
-          <t>HD현대미포</t>
+          <t>농심</t>
         </is>
       </c>
       <c r="E46" s="17" t="n">
@@ -1703,19 +1703,19 @@
     </row>
     <row r="47">
       <c r="A47" s="14" t="n">
-        <v>45365</v>
+        <v>45911</v>
       </c>
       <c r="B47" s="14" t="n">
-        <v>45896</v>
+        <v>45912</v>
       </c>
       <c r="C47" s="15" t="inlineStr">
         <is>
-          <t>010140</t>
+          <t>100090</t>
         </is>
       </c>
       <c r="D47" s="16" t="inlineStr">
         <is>
-          <t>삼성중공업</t>
+          <t>SK오션플랜트</t>
         </is>
       </c>
       <c r="E47" s="17" t="n">
@@ -1727,19 +1727,19 @@
     </row>
     <row r="48">
       <c r="A48" s="14" t="n">
-        <v>45895</v>
+        <v>45908</v>
       </c>
       <c r="B48" s="14" t="n">
-        <v>45895</v>
+        <v>45910</v>
       </c>
       <c r="C48" s="15" t="inlineStr">
         <is>
-          <t>298040</t>
+          <t>075580</t>
         </is>
       </c>
       <c r="D48" s="16" t="inlineStr">
         <is>
-          <t>효성중공업</t>
+          <t>세진중공업</t>
         </is>
       </c>
       <c r="E48" s="17" t="n">
@@ -1751,19 +1751,19 @@
     </row>
     <row r="49">
       <c r="A49" s="14" t="n">
-        <v>45782</v>
+        <v>45908</v>
       </c>
       <c r="B49" s="14" t="n">
-        <v>45895</v>
+        <v>45908</v>
       </c>
       <c r="C49" s="15" t="inlineStr">
         <is>
-          <t>079550</t>
+          <t>290650</t>
         </is>
       </c>
       <c r="D49" s="16" t="inlineStr">
         <is>
-          <t>LIG넥스원</t>
+          <t>엘앤씨바이오</t>
         </is>
       </c>
       <c r="E49" s="17" t="n">
@@ -1775,19 +1775,19 @@
     </row>
     <row r="50">
       <c r="A50" s="14" t="n">
-        <v>45888</v>
+        <v>45898</v>
       </c>
       <c r="B50" s="14" t="n">
-        <v>45888</v>
+        <v>45898</v>
       </c>
       <c r="C50" s="15" t="inlineStr">
         <is>
-          <t>0008Z0</t>
+          <t>082740</t>
         </is>
       </c>
       <c r="D50" s="16" t="inlineStr">
         <is>
-          <t>에스엔시스</t>
+          <t>한화엔진</t>
         </is>
       </c>
       <c r="E50" s="17" t="n">
@@ -1799,19 +1799,19 @@
     </row>
     <row r="51">
       <c r="A51" s="14" t="n">
-        <v>45887</v>
+        <v>45897</v>
       </c>
       <c r="B51" s="14" t="n">
-        <v>45887</v>
+        <v>45897</v>
       </c>
       <c r="C51" s="15" t="inlineStr">
         <is>
-          <t>484590</t>
+          <t>460930</t>
         </is>
       </c>
       <c r="D51" s="16" t="inlineStr">
         <is>
-          <t>삼양컴텍</t>
+          <t>현대힘스</t>
         </is>
       </c>
       <c r="E51" s="17" t="n">
@@ -1823,19 +1823,19 @@
     </row>
     <row r="52">
       <c r="A52" s="14" t="n">
-        <v>45755</v>
+        <v>45897</v>
       </c>
       <c r="B52" s="14" t="n">
-        <v>45883</v>
+        <v>45897</v>
       </c>
       <c r="C52" s="15" t="inlineStr">
         <is>
-          <t>298380</t>
+          <t>009540</t>
         </is>
       </c>
       <c r="D52" s="16" t="inlineStr">
         <is>
-          <t>에이비엘바이오</t>
+          <t>HD한국조선해양</t>
         </is>
       </c>
       <c r="E52" s="17" t="n">
@@ -1847,19 +1847,19 @@
     </row>
     <row r="53">
       <c r="A53" s="14" t="n">
-        <v>45882</v>
+        <v>45896</v>
       </c>
       <c r="B53" s="14" t="n">
-        <v>45882</v>
+        <v>45897</v>
       </c>
       <c r="C53" s="15" t="inlineStr">
         <is>
-          <t>034220</t>
+          <t>010620</t>
         </is>
       </c>
       <c r="D53" s="16" t="inlineStr">
         <is>
-          <t>LG디스플레이</t>
+          <t>HD현대미포</t>
         </is>
       </c>
       <c r="E53" s="17" t="n">
@@ -1871,19 +1871,19 @@
     </row>
     <row r="54">
       <c r="A54" s="14" t="n">
-        <v>45870</v>
+        <v>45895</v>
       </c>
       <c r="B54" s="14" t="n">
-        <v>45876</v>
+        <v>45895</v>
       </c>
       <c r="C54" s="15" t="inlineStr">
         <is>
-          <t>439260</t>
+          <t>298040</t>
         </is>
       </c>
       <c r="D54" s="16" t="inlineStr">
         <is>
-          <t>대한조선</t>
+          <t>효성중공업</t>
         </is>
       </c>
       <c r="E54" s="17" t="n">
@@ -1895,19 +1895,19 @@
     </row>
     <row r="55">
       <c r="A55" s="14" t="n">
-        <v>45785</v>
+        <v>45782</v>
       </c>
       <c r="B55" s="14" t="n">
-        <v>45875</v>
+        <v>45895</v>
       </c>
       <c r="C55" s="15" t="inlineStr">
         <is>
-          <t>278470</t>
+          <t>079550</t>
         </is>
       </c>
       <c r="D55" s="16" t="inlineStr">
         <is>
-          <t>에이피알</t>
+          <t>LIG넥스원</t>
         </is>
       </c>
       <c r="E55" s="17" t="n">
@@ -1919,19 +1919,19 @@
     </row>
     <row r="56">
       <c r="A56" s="14" t="n">
-        <v>45874</v>
+        <v>45888</v>
       </c>
       <c r="B56" s="14" t="n">
-        <v>45874</v>
+        <v>45888</v>
       </c>
       <c r="C56" s="15" t="inlineStr">
         <is>
-          <t>326030</t>
+          <t>0008Z0</t>
         </is>
       </c>
       <c r="D56" s="16" t="inlineStr">
         <is>
-          <t>SK바이오팜</t>
+          <t>에스엔시스</t>
         </is>
       </c>
       <c r="E56" s="17" t="n">
@@ -1943,19 +1943,19 @@
     </row>
     <row r="57">
       <c r="A57" s="14" t="n">
-        <v>45699</v>
+        <v>45887</v>
       </c>
       <c r="B57" s="14" t="n">
-        <v>45870</v>
+        <v>45887</v>
       </c>
       <c r="C57" s="15" t="inlineStr">
         <is>
-          <t>012450</t>
+          <t>484590</t>
         </is>
       </c>
       <c r="D57" s="16" t="inlineStr">
         <is>
-          <t>한화에어로스페이스</t>
+          <t>삼양컴텍</t>
         </is>
       </c>
       <c r="E57" s="17" t="n">
@@ -1967,19 +1967,19 @@
     </row>
     <row r="58">
       <c r="A58" s="14" t="n">
-        <v>45700</v>
+        <v>45755</v>
       </c>
       <c r="B58" s="14" t="n">
-        <v>45869</v>
+        <v>45883</v>
       </c>
       <c r="C58" s="15" t="inlineStr">
         <is>
-          <t>272210</t>
+          <t>298380</t>
         </is>
       </c>
       <c r="D58" s="16" t="inlineStr">
         <is>
-          <t>한화시스템</t>
+          <t>에이비엘바이오</t>
         </is>
       </c>
       <c r="E58" s="17" t="n">
@@ -1991,19 +1991,19 @@
     </row>
     <row r="59">
       <c r="A59" s="14" t="n">
-        <v>45772</v>
+        <v>45882</v>
       </c>
       <c r="B59" s="14" t="n">
-        <v>45868</v>
+        <v>45882</v>
       </c>
       <c r="C59" s="15" t="inlineStr">
         <is>
-          <t>009830</t>
+          <t>034220</t>
         </is>
       </c>
       <c r="D59" s="16" t="inlineStr">
         <is>
-          <t>한화솔루션</t>
+          <t>LG디스플레이</t>
         </is>
       </c>
       <c r="E59" s="17" t="n">
@@ -2015,19 +2015,19 @@
     </row>
     <row r="60">
       <c r="A60" s="14" t="n">
-        <v>45868</v>
+        <v>45870</v>
       </c>
       <c r="B60" s="14" t="n">
-        <v>45868</v>
+        <v>45876</v>
       </c>
       <c r="C60" s="15" t="inlineStr">
         <is>
-          <t>009150</t>
+          <t>439260</t>
         </is>
       </c>
       <c r="D60" s="16" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>대한조선</t>
         </is>
       </c>
       <c r="E60" s="17" t="n">
@@ -2039,19 +2039,19 @@
     </row>
     <row r="61">
       <c r="A61" s="14" t="n">
-        <v>45867</v>
+        <v>45785</v>
       </c>
       <c r="B61" s="14" t="n">
-        <v>45867</v>
+        <v>45875</v>
       </c>
       <c r="C61" s="15" t="inlineStr">
         <is>
-          <t>489790</t>
+          <t>278470</t>
         </is>
       </c>
       <c r="D61" s="16" t="inlineStr">
         <is>
-          <t>한화비전</t>
+          <t>에이피알</t>
         </is>
       </c>
       <c r="E61" s="17" t="n">
@@ -2063,19 +2063,19 @@
     </row>
     <row r="62">
       <c r="A62" s="14" t="n">
-        <v>45862</v>
+        <v>45874</v>
       </c>
       <c r="B62" s="14" t="n">
-        <v>45867</v>
+        <v>45874</v>
       </c>
       <c r="C62" s="15" t="inlineStr">
         <is>
-          <t>042670</t>
+          <t>326030</t>
         </is>
       </c>
       <c r="D62" s="16" t="inlineStr">
         <is>
-          <t>HD현대인프라코어</t>
+          <t>SK바이오팜</t>
         </is>
       </c>
       <c r="E62" s="17" t="n">
@@ -2087,19 +2087,19 @@
     </row>
     <row r="63">
       <c r="A63" s="14" t="n">
-        <v>45861</v>
+        <v>45699</v>
       </c>
       <c r="B63" s="14" t="n">
-        <v>45861</v>
+        <v>45870</v>
       </c>
       <c r="C63" s="15" t="inlineStr">
         <is>
-          <t>484120</t>
+          <t>012450</t>
         </is>
       </c>
       <c r="D63" s="16" t="inlineStr">
         <is>
-          <t>도우인시스</t>
+          <t>한화에어로스페이스</t>
         </is>
       </c>
       <c r="E63" s="17" t="n">
@@ -2111,19 +2111,19 @@
     </row>
     <row r="64">
       <c r="A64" s="14" t="n">
-        <v>45846</v>
+        <v>45700</v>
       </c>
       <c r="B64" s="14" t="n">
-        <v>45861</v>
+        <v>45869</v>
       </c>
       <c r="C64" s="15" t="inlineStr">
         <is>
-          <t>008970</t>
+          <t>272210</t>
         </is>
       </c>
       <c r="D64" s="16" t="inlineStr">
         <is>
-          <t>KBI동양철관</t>
+          <t>한화시스템</t>
         </is>
       </c>
       <c r="E64" s="17" t="n">
@@ -2135,19 +2135,19 @@
     </row>
     <row r="65">
       <c r="A65" s="14" t="n">
-        <v>45860</v>
+        <v>45772</v>
       </c>
       <c r="B65" s="14" t="n">
-        <v>45860</v>
+        <v>45868</v>
       </c>
       <c r="C65" s="15" t="inlineStr">
         <is>
-          <t>037270</t>
+          <t>009830</t>
         </is>
       </c>
       <c r="D65" s="16" t="inlineStr">
         <is>
-          <t>YG PLUS</t>
+          <t>한화솔루션</t>
         </is>
       </c>
       <c r="E65" s="17" t="n">
@@ -2159,19 +2159,19 @@
     </row>
     <row r="66">
       <c r="A66" s="14" t="n">
-        <v>45856</v>
+        <v>45868</v>
       </c>
       <c r="B66" s="14" t="n">
-        <v>45856</v>
+        <v>45868</v>
       </c>
       <c r="C66" s="15" t="inlineStr">
         <is>
-          <t>141080</t>
+          <t>009150</t>
         </is>
       </c>
       <c r="D66" s="16" t="inlineStr">
         <is>
-          <t>리가켐바이오</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="E66" s="17" t="n">
@@ -2183,19 +2183,19 @@
     </row>
     <row r="67">
       <c r="A67" s="14" t="n">
-        <v>45854</v>
+        <v>45867</v>
       </c>
       <c r="B67" s="14" t="n">
-        <v>45854</v>
+        <v>45867</v>
       </c>
       <c r="C67" s="15" t="inlineStr">
         <is>
-          <t>294570</t>
+          <t>489790</t>
         </is>
       </c>
       <c r="D67" s="16" t="inlineStr">
         <is>
-          <t>쿠콘</t>
+          <t>한화비전</t>
         </is>
       </c>
       <c r="E67" s="17" t="n">
@@ -2207,19 +2207,19 @@
     </row>
     <row r="68">
       <c r="A68" s="14" t="n">
-        <v>45854</v>
+        <v>45862</v>
       </c>
       <c r="B68" s="14" t="n">
-        <v>45854</v>
+        <v>45867</v>
       </c>
       <c r="C68" s="15" t="inlineStr">
         <is>
-          <t>441270</t>
+          <t>042670</t>
         </is>
       </c>
       <c r="D68" s="16" t="inlineStr">
         <is>
-          <t>파인엠텍</t>
+          <t>HD현대인프라코어</t>
         </is>
       </c>
       <c r="E68" s="17" t="n">
@@ -2231,19 +2231,19 @@
     </row>
     <row r="69">
       <c r="A69" s="14" t="n">
-        <v>45849</v>
+        <v>45861</v>
       </c>
       <c r="B69" s="14" t="n">
-        <v>45849</v>
+        <v>45861</v>
       </c>
       <c r="C69" s="15" t="inlineStr">
         <is>
-          <t>402340</t>
+          <t>484120</t>
         </is>
       </c>
       <c r="D69" s="16" t="inlineStr">
         <is>
-          <t>SK스퀘어</t>
+          <t>도우인시스</t>
         </is>
       </c>
       <c r="E69" s="17" t="n">
@@ -2255,19 +2255,19 @@
     </row>
     <row r="70">
       <c r="A70" s="14" t="n">
-        <v>45841</v>
+        <v>45846</v>
       </c>
       <c r="B70" s="14" t="n">
-        <v>45842</v>
+        <v>45861</v>
       </c>
       <c r="C70" s="15" t="inlineStr">
         <is>
-          <t>005490</t>
+          <t>008970</t>
         </is>
       </c>
       <c r="D70" s="16" t="inlineStr">
         <is>
-          <t>POSCO홀딩스</t>
+          <t>KBI동양철관</t>
         </is>
       </c>
       <c r="E70" s="17" t="n">
@@ -2279,19 +2279,19 @@
     </row>
     <row r="71">
       <c r="A71" s="14" t="n">
-        <v>45840</v>
+        <v>45860</v>
       </c>
       <c r="B71" s="14" t="n">
-        <v>45840</v>
+        <v>45860</v>
       </c>
       <c r="C71" s="15" t="inlineStr">
         <is>
-          <t>267270</t>
+          <t>037270</t>
         </is>
       </c>
       <c r="D71" s="16" t="inlineStr">
         <is>
-          <t>HD현대건설기계</t>
+          <t>YG PLUS</t>
         </is>
       </c>
       <c r="E71" s="17" t="n">
@@ -2303,19 +2303,19 @@
     </row>
     <row r="72">
       <c r="A72" s="14" t="n">
-        <v>45839</v>
+        <v>45856</v>
       </c>
       <c r="B72" s="14" t="n">
-        <v>45839</v>
+        <v>45856</v>
       </c>
       <c r="C72" s="15" t="inlineStr">
         <is>
-          <t>000880</t>
+          <t>141080</t>
         </is>
       </c>
       <c r="D72" s="16" t="inlineStr">
         <is>
-          <t>한화</t>
+          <t>리가켐바이오</t>
         </is>
       </c>
       <c r="E72" s="17" t="n">
@@ -2327,19 +2327,19 @@
     </row>
     <row r="73">
       <c r="A73" s="14" t="n">
-        <v>43997</v>
+        <v>45854</v>
       </c>
       <c r="B73" s="14" t="n">
-        <v>45839</v>
+        <v>45854</v>
       </c>
       <c r="C73" s="15" t="inlineStr">
         <is>
-          <t>034730</t>
+          <t>294570</t>
         </is>
       </c>
       <c r="D73" s="16" t="inlineStr">
         <is>
-          <t>SK</t>
+          <t>쿠콘</t>
         </is>
       </c>
       <c r="E73" s="17" t="n">
@@ -2351,25 +2351,169 @@
     </row>
     <row r="74">
       <c r="A74" s="14" t="n">
+        <v>45854</v>
+      </c>
+      <c r="B74" s="14" t="n">
+        <v>45854</v>
+      </c>
+      <c r="C74" s="15" t="inlineStr">
+        <is>
+          <t>441270</t>
+        </is>
+      </c>
+      <c r="D74" s="16" t="inlineStr">
+        <is>
+          <t>파인엠텍</t>
+        </is>
+      </c>
+      <c r="E74" s="17" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F74" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="14" t="n">
+        <v>45849</v>
+      </c>
+      <c r="B75" s="14" t="n">
+        <v>45849</v>
+      </c>
+      <c r="C75" s="15" t="inlineStr">
+        <is>
+          <t>402340</t>
+        </is>
+      </c>
+      <c r="D75" s="16" t="inlineStr">
+        <is>
+          <t>SK스퀘어</t>
+        </is>
+      </c>
+      <c r="E75" s="17" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F75" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="14" t="n">
+        <v>45841</v>
+      </c>
+      <c r="B76" s="14" t="n">
+        <v>45842</v>
+      </c>
+      <c r="C76" s="15" t="inlineStr">
+        <is>
+          <t>005490</t>
+        </is>
+      </c>
+      <c r="D76" s="16" t="inlineStr">
+        <is>
+          <t>POSCO홀딩스</t>
+        </is>
+      </c>
+      <c r="E76" s="17" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F76" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="14" t="n">
+        <v>45840</v>
+      </c>
+      <c r="B77" s="14" t="n">
+        <v>45840</v>
+      </c>
+      <c r="C77" s="15" t="inlineStr">
+        <is>
+          <t>267270</t>
+        </is>
+      </c>
+      <c r="D77" s="16" t="inlineStr">
+        <is>
+          <t>HD현대건설기계</t>
+        </is>
+      </c>
+      <c r="E77" s="17" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F77" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="14" t="n">
+        <v>45839</v>
+      </c>
+      <c r="B78" s="14" t="n">
+        <v>45839</v>
+      </c>
+      <c r="C78" s="15" t="inlineStr">
+        <is>
+          <t>000880</t>
+        </is>
+      </c>
+      <c r="D78" s="16" t="inlineStr">
+        <is>
+          <t>한화</t>
+        </is>
+      </c>
+      <c r="E78" s="17" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F78" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="14" t="n">
+        <v>43997</v>
+      </c>
+      <c r="B79" s="14" t="n">
+        <v>45839</v>
+      </c>
+      <c r="C79" s="15" t="inlineStr">
+        <is>
+          <t>034730</t>
+        </is>
+      </c>
+      <c r="D79" s="16" t="inlineStr">
+        <is>
+          <t>SK</t>
+        </is>
+      </c>
+      <c r="E79" s="17" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F79" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="14" t="n">
         <v>45838</v>
       </c>
-      <c r="B74" s="14" t="n">
+      <c r="B80" s="14" t="n">
         <v>45839</v>
       </c>
-      <c r="C74" s="15" t="inlineStr">
+      <c r="C80" s="15" t="inlineStr">
         <is>
           <t>096770</t>
         </is>
       </c>
-      <c r="D74" s="16" t="inlineStr">
+      <c r="D80" s="16" t="inlineStr">
         <is>
           <t>SK이노베이션</t>
         </is>
       </c>
-      <c r="E74" s="17" t="n">
-        <v>5000</v>
-      </c>
-      <c r="F74" s="18" t="n">
+      <c r="E80" s="17" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F80" s="18" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: Add CLAUDE.md for future Claude Code instances
- Comprehensive system documentation for S12 Trading System
- Architecture overview with data flow
- Commands for daily operations, real-time monitoring, and testing
- Technical details (tick price calculation, alert logic, Excel formatting)
- Troubleshooting guide and known issues
- Include .claude/ settings and recent logs

🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/turnover_universe.xlsx
+++ b/output/turnover_universe.xlsx
@@ -573,7 +573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H80"/>
+  <dimension ref="A1:H81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -617,7 +617,7 @@
       </c>
       <c r="H1" s="13" t="inlineStr">
         <is>
-          <t>최종 업데이트: 2025-10-29</t>
+          <t>최종 업데이트: 2025-10-30</t>
         </is>
       </c>
     </row>
@@ -626,7 +626,7 @@
         <v>45942</v>
       </c>
       <c r="B2" s="14" t="n">
-        <v>45959</v>
+        <v>45960</v>
       </c>
       <c r="C2" s="15" t="inlineStr">
         <is>
@@ -639,10 +639,10 @@
         </is>
       </c>
       <c r="E2" s="17" t="n">
-        <v>34789.85</v>
+        <v>61144.41</v>
       </c>
       <c r="F2" s="18" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3">
@@ -650,7 +650,7 @@
         <v>45942</v>
       </c>
       <c r="B3" s="14" t="n">
-        <v>45959</v>
+        <v>45960</v>
       </c>
       <c r="C3" s="15" t="inlineStr">
         <is>
@@ -663,10 +663,10 @@
         </is>
       </c>
       <c r="E3" s="17" t="n">
-        <v>52358.47</v>
+        <v>48948.26</v>
       </c>
       <c r="F3" s="18" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4">
@@ -674,7 +674,7 @@
         <v>45942</v>
       </c>
       <c r="B4" s="14" t="n">
-        <v>45959</v>
+        <v>45960</v>
       </c>
       <c r="C4" s="15" t="inlineStr">
         <is>
@@ -687,10 +687,10 @@
         </is>
       </c>
       <c r="E4" s="17" t="n">
-        <v>39513.58</v>
+        <v>21336.9</v>
       </c>
       <c r="F4" s="18" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5">
@@ -698,7 +698,7 @@
         <v>45604</v>
       </c>
       <c r="B5" s="14" t="n">
-        <v>45959</v>
+        <v>45960</v>
       </c>
       <c r="C5" s="15" t="inlineStr">
         <is>
@@ -711,10 +711,10 @@
         </is>
       </c>
       <c r="E5" s="17" t="n">
-        <v>15944.28</v>
+        <v>24575.94</v>
       </c>
       <c r="F5" s="18" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
@@ -722,7 +722,7 @@
         <v>45942</v>
       </c>
       <c r="B6" s="14" t="n">
-        <v>45959</v>
+        <v>45960</v>
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
@@ -735,10 +735,10 @@
         </is>
       </c>
       <c r="E6" s="17" t="n">
-        <v>12265.68</v>
+        <v>7437.190000000001</v>
       </c>
       <c r="F6" s="18" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7">
@@ -746,7 +746,7 @@
         <v>45730</v>
       </c>
       <c r="B7" s="14" t="n">
-        <v>45959</v>
+        <v>45960</v>
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
@@ -759,10 +759,10 @@
         </is>
       </c>
       <c r="E7" s="17" t="n">
-        <v>13351.78</v>
+        <v>10935.75</v>
       </c>
       <c r="F7" s="18" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8">
@@ -770,7 +770,7 @@
         <v>45942</v>
       </c>
       <c r="B8" s="14" t="n">
-        <v>45959</v>
+        <v>45960</v>
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
@@ -783,10 +783,10 @@
         </is>
       </c>
       <c r="E8" s="17" t="n">
-        <v>9485.610000000001</v>
+        <v>6500.89</v>
       </c>
       <c r="F8" s="18" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9">
@@ -794,7 +794,7 @@
         <v>45833</v>
       </c>
       <c r="B9" s="14" t="n">
-        <v>45959</v>
+        <v>45960</v>
       </c>
       <c r="C9" s="15" t="inlineStr">
         <is>
@@ -807,10 +807,10 @@
         </is>
       </c>
       <c r="E9" s="17" t="n">
-        <v>12484.9</v>
+        <v>18592.32</v>
       </c>
       <c r="F9" s="18" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10">
@@ -818,7 +818,7 @@
         <v>45947</v>
       </c>
       <c r="B10" s="14" t="n">
-        <v>45958</v>
+        <v>45960</v>
       </c>
       <c r="C10" s="15" t="inlineStr">
         <is>
@@ -831,31 +831,31 @@
         </is>
       </c>
       <c r="E10" s="17" t="n">
-        <v>8493.91</v>
+        <v>6340.43</v>
       </c>
       <c r="F10" s="18" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
-        <v>45856</v>
+        <v>45365</v>
       </c>
       <c r="B11" s="14" t="n">
-        <v>45958</v>
+        <v>45960</v>
       </c>
       <c r="C11" s="15" t="inlineStr">
         <is>
-          <t>003670</t>
+          <t>010140</t>
         </is>
       </c>
       <c r="D11" s="16" t="inlineStr">
         <is>
-          <t>포스코퓨처엠</t>
+          <t>삼성중공업</t>
         </is>
       </c>
       <c r="E11" s="17" t="n">
-        <v>5493.64</v>
+        <v>9886.030000000001</v>
       </c>
       <c r="F11" s="18" t="n">
         <v>5</v>
@@ -863,23 +863,23 @@
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
-        <v>45874</v>
+        <v>44876</v>
       </c>
       <c r="B12" s="14" t="n">
-        <v>45957</v>
+        <v>45960</v>
       </c>
       <c r="C12" s="15" t="inlineStr">
         <is>
-          <t>247540</t>
+          <t>035720</t>
         </is>
       </c>
       <c r="D12" s="16" t="inlineStr">
         <is>
-          <t>에코프로비엠</t>
+          <t>카카오</t>
         </is>
       </c>
       <c r="E12" s="17" t="n">
-        <v>12071.61</v>
+        <v>7350.05</v>
       </c>
       <c r="F12" s="18" t="n">
         <v>5</v>
@@ -887,74 +887,74 @@
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
-        <v>45365</v>
+        <v>45856</v>
       </c>
       <c r="B13" s="14" t="n">
-        <v>45959</v>
+        <v>45958</v>
       </c>
       <c r="C13" s="15" t="inlineStr">
         <is>
-          <t>010140</t>
+          <t>003670</t>
         </is>
       </c>
       <c r="D13" s="16" t="inlineStr">
         <is>
-          <t>삼성중공업</t>
+          <t>포스코퓨처엠</t>
         </is>
       </c>
       <c r="E13" s="17" t="n">
-        <v>9568.76</v>
+        <v>5493.64</v>
       </c>
       <c r="F13" s="18" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
-        <v>44876</v>
+        <v>45874</v>
       </c>
       <c r="B14" s="14" t="n">
-        <v>45959</v>
+        <v>45957</v>
       </c>
       <c r="C14" s="15" t="inlineStr">
         <is>
-          <t>035720</t>
+          <t>247540</t>
         </is>
       </c>
       <c r="D14" s="16" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>에코프로비엠</t>
         </is>
       </c>
       <c r="E14" s="17" t="n">
-        <v>16671.6</v>
+        <v>12071.61</v>
       </c>
       <c r="F14" s="18" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
-        <v>45947</v>
+        <v>45946</v>
       </c>
       <c r="B15" s="14" t="n">
-        <v>45952</v>
+        <v>45960</v>
       </c>
       <c r="C15" s="15" t="inlineStr">
         <is>
-          <t>051910</t>
+          <t>373220</t>
         </is>
       </c>
       <c r="D15" s="16" t="inlineStr">
         <is>
-          <t>LG화학</t>
+          <t>LG에너지솔루션</t>
         </is>
       </c>
       <c r="E15" s="17" t="n">
-        <v>9404.630000000001</v>
+        <v>5356.72</v>
       </c>
       <c r="F15" s="18" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16">
@@ -962,20 +962,20 @@
         <v>45947</v>
       </c>
       <c r="B16" s="14" t="n">
-        <v>45949</v>
+        <v>45960</v>
       </c>
       <c r="C16" s="15" t="inlineStr">
         <is>
-          <t>450080</t>
+          <t>066970</t>
         </is>
       </c>
       <c r="D16" s="16" t="inlineStr">
         <is>
-          <t>에코프로머티</t>
+          <t>엘앤에프</t>
         </is>
       </c>
       <c r="E16" s="17" t="n">
-        <v>7222.29</v>
+        <v>5207</v>
       </c>
       <c r="F16" s="18" t="n">
         <v>3</v>
@@ -983,23 +983,23 @@
     </row>
     <row r="17">
       <c r="A17" s="14" t="n">
-        <v>45946</v>
+        <v>45947</v>
       </c>
       <c r="B17" s="14" t="n">
-        <v>45949</v>
+        <v>45952</v>
       </c>
       <c r="C17" s="15" t="inlineStr">
         <is>
-          <t>373220</t>
+          <t>051910</t>
         </is>
       </c>
       <c r="D17" s="16" t="inlineStr">
         <is>
-          <t>LG에너지솔루션</t>
+          <t>LG화학</t>
         </is>
       </c>
       <c r="E17" s="17" t="n">
-        <v>6561.16</v>
+        <v>9404.630000000001</v>
       </c>
       <c r="F17" s="18" t="n">
         <v>3</v>
@@ -1007,23 +1007,23 @@
     </row>
     <row r="18">
       <c r="A18" s="14" t="n">
-        <v>45853</v>
+        <v>45947</v>
       </c>
       <c r="B18" s="14" t="n">
         <v>45949</v>
       </c>
       <c r="C18" s="15" t="inlineStr">
         <is>
-          <t>015760</t>
+          <t>450080</t>
         </is>
       </c>
       <c r="D18" s="16" t="inlineStr">
         <is>
-          <t>한국전력</t>
+          <t>에코프로머티</t>
         </is>
       </c>
       <c r="E18" s="17" t="n">
-        <v>6619.35</v>
+        <v>7222.29</v>
       </c>
       <c r="F18" s="18" t="n">
         <v>3</v>
@@ -1031,47 +1031,47 @@
     </row>
     <row r="19">
       <c r="A19" s="14" t="n">
-        <v>45958</v>
+        <v>45853</v>
       </c>
       <c r="B19" s="14" t="n">
-        <v>45959</v>
+        <v>45949</v>
       </c>
       <c r="C19" s="15" t="inlineStr">
         <is>
-          <t>336260</t>
+          <t>015760</t>
         </is>
       </c>
       <c r="D19" s="16" t="inlineStr">
         <is>
-          <t>두산퓨얼셀</t>
+          <t>한국전력</t>
         </is>
       </c>
       <c r="E19" s="17" t="n">
-        <v>5907.51</v>
+        <v>6619.35</v>
       </c>
       <c r="F19" s="18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="14" t="n">
-        <v>45957</v>
+        <v>45942</v>
       </c>
       <c r="B20" s="14" t="n">
-        <v>45959</v>
+        <v>45960</v>
       </c>
       <c r="C20" s="15" t="inlineStr">
         <is>
-          <t>000720</t>
+          <t>108490</t>
         </is>
       </c>
       <c r="D20" s="16" t="inlineStr">
         <is>
-          <t>현대건설</t>
+          <t>로보티즈</t>
         </is>
       </c>
       <c r="E20" s="17" t="n">
-        <v>7859.2</v>
+        <v>6265.45</v>
       </c>
       <c r="F20" s="18" t="n">
         <v>2</v>
@@ -1079,23 +1079,23 @@
     </row>
     <row r="21">
       <c r="A21" s="14" t="n">
-        <v>45650</v>
+        <v>45942</v>
       </c>
       <c r="B21" s="14" t="n">
-        <v>45957</v>
+        <v>45960</v>
       </c>
       <c r="C21" s="15" t="inlineStr">
         <is>
-          <t>196170</t>
+          <t>005935</t>
         </is>
       </c>
       <c r="D21" s="16" t="inlineStr">
         <is>
-          <t>알테오젠</t>
+          <t>삼성전자우</t>
         </is>
       </c>
       <c r="E21" s="17" t="n">
-        <v>6894.2</v>
+        <v>6234.82</v>
       </c>
       <c r="F21" s="18" t="n">
         <v>2</v>
@@ -1103,23 +1103,23 @@
     </row>
     <row r="22">
       <c r="A22" s="14" t="n">
-        <v>45876</v>
+        <v>45700</v>
       </c>
       <c r="B22" s="14" t="n">
-        <v>45957</v>
+        <v>45960</v>
       </c>
       <c r="C22" s="15" t="inlineStr">
         <is>
-          <t>097230</t>
+          <t>272210</t>
         </is>
       </c>
       <c r="D22" s="16" t="inlineStr">
         <is>
-          <t>HJ중공업</t>
+          <t>한화시스템</t>
         </is>
       </c>
       <c r="E22" s="17" t="n">
-        <v>6016.41</v>
+        <v>14791.78</v>
       </c>
       <c r="F22" s="18" t="n">
         <v>2</v>
@@ -1127,23 +1127,23 @@
     </row>
     <row r="23">
       <c r="A23" s="14" t="n">
-        <v>45694</v>
+        <v>45958</v>
       </c>
       <c r="B23" s="14" t="n">
-        <v>45952</v>
+        <v>45959</v>
       </c>
       <c r="C23" s="15" t="inlineStr">
         <is>
-          <t>064350</t>
+          <t>336260</t>
         </is>
       </c>
       <c r="D23" s="16" t="inlineStr">
         <is>
-          <t>현대로템</t>
+          <t>두산퓨얼셀</t>
         </is>
       </c>
       <c r="E23" s="17" t="n">
-        <v>6133.97</v>
+        <v>5907.51</v>
       </c>
       <c r="F23" s="18" t="n">
         <v>2</v>
@@ -1151,23 +1151,23 @@
     </row>
     <row r="24">
       <c r="A24" s="14" t="n">
-        <v>45947</v>
+        <v>45957</v>
       </c>
       <c r="B24" s="14" t="n">
-        <v>45949</v>
+        <v>45959</v>
       </c>
       <c r="C24" s="15" t="inlineStr">
         <is>
-          <t>066970</t>
+          <t>000720</t>
         </is>
       </c>
       <c r="D24" s="16" t="inlineStr">
         <is>
-          <t>엘앤에프</t>
+          <t>현대건설</t>
         </is>
       </c>
       <c r="E24" s="17" t="n">
-        <v>5810.01</v>
+        <v>7859.2</v>
       </c>
       <c r="F24" s="18" t="n">
         <v>2</v>
@@ -1175,23 +1175,23 @@
     </row>
     <row r="25">
       <c r="A25" s="14" t="n">
-        <v>45947</v>
+        <v>45650</v>
       </c>
       <c r="B25" s="14" t="n">
-        <v>45949</v>
+        <v>45957</v>
       </c>
       <c r="C25" s="15" t="inlineStr">
         <is>
-          <t>000150</t>
+          <t>196170</t>
         </is>
       </c>
       <c r="D25" s="16" t="inlineStr">
         <is>
-          <t>두산</t>
+          <t>알테오젠</t>
         </is>
       </c>
       <c r="E25" s="17" t="n">
-        <v>5742.17</v>
+        <v>6894.2</v>
       </c>
       <c r="F25" s="18" t="n">
         <v>2</v>
@@ -1199,23 +1199,23 @@
     </row>
     <row r="26">
       <c r="A26" s="14" t="n">
-        <v>45916</v>
+        <v>45876</v>
       </c>
       <c r="B26" s="14" t="n">
-        <v>45945</v>
+        <v>45957</v>
       </c>
       <c r="C26" s="15" t="inlineStr">
         <is>
-          <t>125490</t>
+          <t>097230</t>
         </is>
       </c>
       <c r="D26" s="16" t="inlineStr">
         <is>
-          <t>한라캐스트</t>
+          <t>HJ중공업</t>
         </is>
       </c>
       <c r="E26" s="17" t="n">
-        <v>5614.12</v>
+        <v>6016.41</v>
       </c>
       <c r="F26" s="18" t="n">
         <v>2</v>
@@ -1223,95 +1223,95 @@
     </row>
     <row r="27">
       <c r="A27" s="14" t="n">
-        <v>45959</v>
+        <v>45694</v>
       </c>
       <c r="B27" s="14" t="n">
-        <v>45959</v>
+        <v>45952</v>
       </c>
       <c r="C27" s="15" t="inlineStr">
         <is>
-          <t>001440</t>
+          <t>064350</t>
         </is>
       </c>
       <c r="D27" s="16" t="inlineStr">
         <is>
-          <t>대한전선</t>
+          <t>현대로템</t>
         </is>
       </c>
       <c r="E27" s="17" t="n">
-        <v>5087.57</v>
+        <v>6133.97</v>
       </c>
       <c r="F27" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="14" t="n">
-        <v>45958</v>
+        <v>45947</v>
       </c>
       <c r="B28" s="14" t="n">
-        <v>45958</v>
+        <v>45949</v>
       </c>
       <c r="C28" s="15" t="inlineStr">
         <is>
-          <t>011790</t>
+          <t>000150</t>
         </is>
       </c>
       <c r="D28" s="16" t="inlineStr">
         <is>
-          <t>SKC</t>
+          <t>두산</t>
         </is>
       </c>
       <c r="E28" s="17" t="n">
-        <v>5001.6</v>
+        <v>5742.17</v>
       </c>
       <c r="F28" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="14" t="n">
-        <v>45957</v>
+        <v>45916</v>
       </c>
       <c r="B29" s="14" t="n">
-        <v>45957</v>
+        <v>45945</v>
       </c>
       <c r="C29" s="15" t="inlineStr">
         <is>
-          <t>128940</t>
+          <t>125490</t>
         </is>
       </c>
       <c r="D29" s="16" t="inlineStr">
         <is>
-          <t>한미약품</t>
+          <t>한라캐스트</t>
         </is>
       </c>
       <c r="E29" s="17" t="n">
-        <v>7324.5</v>
+        <v>5614.12</v>
       </c>
       <c r="F29" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="14" t="n">
-        <v>45957</v>
+        <v>45960</v>
       </c>
       <c r="B30" s="14" t="n">
-        <v>45957</v>
+        <v>45960</v>
       </c>
       <c r="C30" s="15" t="inlineStr">
         <is>
-          <t>352820</t>
+          <t>000270</t>
         </is>
       </c>
       <c r="D30" s="16" t="inlineStr">
         <is>
-          <t>하이브</t>
+          <t>기아</t>
         </is>
       </c>
       <c r="E30" s="17" t="n">
-        <v>5473.690000000001</v>
+        <v>5648.01</v>
       </c>
       <c r="F30" s="18" t="n">
         <v>1</v>
@@ -1319,23 +1319,23 @@
     </row>
     <row r="31">
       <c r="A31" s="14" t="n">
-        <v>45951</v>
+        <v>45959</v>
       </c>
       <c r="B31" s="14" t="n">
-        <v>45951</v>
+        <v>45959</v>
       </c>
       <c r="C31" s="15" t="inlineStr">
         <is>
-          <t>090710</t>
+          <t>001440</t>
         </is>
       </c>
       <c r="D31" s="16" t="inlineStr">
         <is>
-          <t>휴림로봇</t>
+          <t>대한전선</t>
         </is>
       </c>
       <c r="E31" s="17" t="n">
-        <v>7343.57</v>
+        <v>5087.57</v>
       </c>
       <c r="F31" s="18" t="n">
         <v>1</v>
@@ -1343,23 +1343,23 @@
     </row>
     <row r="32">
       <c r="A32" s="14" t="n">
-        <v>45943</v>
+        <v>45958</v>
       </c>
       <c r="B32" s="14" t="n">
-        <v>45943</v>
+        <v>45958</v>
       </c>
       <c r="C32" s="15" t="inlineStr">
         <is>
-          <t>466100</t>
+          <t>011790</t>
         </is>
       </c>
       <c r="D32" s="16" t="inlineStr">
         <is>
-          <t>클로봇</t>
+          <t>SKC</t>
         </is>
       </c>
       <c r="E32" s="17" t="n">
-        <v>6494.860000000001</v>
+        <v>5001.6</v>
       </c>
       <c r="F32" s="18" t="n">
         <v>1</v>
@@ -1367,23 +1367,23 @@
     </row>
     <row r="33">
       <c r="A33" s="14" t="n">
-        <v>45942</v>
+        <v>45957</v>
       </c>
       <c r="B33" s="14" t="n">
-        <v>45942</v>
+        <v>45957</v>
       </c>
       <c r="C33" s="15" t="inlineStr">
         <is>
-          <t>108490</t>
+          <t>128940</t>
         </is>
       </c>
       <c r="D33" s="16" t="inlineStr">
         <is>
-          <t>로보티즈</t>
+          <t>한미약품</t>
         </is>
       </c>
       <c r="E33" s="17" t="n">
-        <v>8159.77</v>
+        <v>7324.5</v>
       </c>
       <c r="F33" s="18" t="n">
         <v>1</v>
@@ -1391,23 +1391,23 @@
     </row>
     <row r="34">
       <c r="A34" s="14" t="n">
-        <v>45942</v>
+        <v>45957</v>
       </c>
       <c r="B34" s="14" t="n">
-        <v>45942</v>
+        <v>45957</v>
       </c>
       <c r="C34" s="15" t="inlineStr">
         <is>
-          <t>005935</t>
+          <t>352820</t>
         </is>
       </c>
       <c r="D34" s="16" t="inlineStr">
         <is>
-          <t>삼성전자우</t>
+          <t>하이브</t>
         </is>
       </c>
       <c r="E34" s="17" t="n">
-        <v>5438.03</v>
+        <v>5473.690000000001</v>
       </c>
       <c r="F34" s="18" t="n">
         <v>1</v>
@@ -1415,23 +1415,23 @@
     </row>
     <row r="35">
       <c r="A35" s="14" t="n">
-        <v>44512</v>
+        <v>45951</v>
       </c>
       <c r="B35" s="14" t="n">
-        <v>45929</v>
+        <v>45951</v>
       </c>
       <c r="C35" s="15" t="inlineStr">
         <is>
-          <t>249420</t>
+          <t>090710</t>
         </is>
       </c>
       <c r="D35" s="16" t="inlineStr">
         <is>
-          <t>일동제약</t>
+          <t>휴림로봇</t>
         </is>
       </c>
       <c r="E35" s="17" t="n">
-        <v>9183</v>
+        <v>7343.57</v>
       </c>
       <c r="F35" s="18" t="n">
         <v>1</v>
@@ -1439,23 +1439,23 @@
     </row>
     <row r="36">
       <c r="A36" s="14" t="n">
-        <v>45849</v>
+        <v>45943</v>
       </c>
       <c r="B36" s="14" t="n">
-        <v>45929</v>
+        <v>45943</v>
       </c>
       <c r="C36" s="15" t="inlineStr">
         <is>
-          <t>041190</t>
+          <t>466100</t>
         </is>
       </c>
       <c r="D36" s="16" t="inlineStr">
         <is>
-          <t>우리기술투자</t>
+          <t>클로봇</t>
         </is>
       </c>
       <c r="E36" s="17" t="n">
-        <v>5517</v>
+        <v>6494.860000000001</v>
       </c>
       <c r="F36" s="18" t="n">
         <v>1</v>
@@ -1463,23 +1463,23 @@
     </row>
     <row r="37">
       <c r="A37" s="14" t="n">
-        <v>45849</v>
+        <v>44512</v>
       </c>
       <c r="B37" s="14" t="n">
-        <v>45926</v>
+        <v>45929</v>
       </c>
       <c r="C37" s="15" t="inlineStr">
         <is>
-          <t>060250</t>
+          <t>249420</t>
         </is>
       </c>
       <c r="D37" s="16" t="inlineStr">
         <is>
-          <t>NHN KCP</t>
+          <t>일동제약</t>
         </is>
       </c>
       <c r="E37" s="17" t="n">
-        <v>9171</v>
+        <v>9183</v>
       </c>
       <c r="F37" s="18" t="n">
         <v>1</v>
@@ -1487,23 +1487,23 @@
     </row>
     <row r="38">
       <c r="A38" s="14" t="n">
-        <v>45925</v>
+        <v>45849</v>
       </c>
       <c r="B38" s="14" t="n">
-        <v>45925</v>
+        <v>45929</v>
       </c>
       <c r="C38" s="15" t="inlineStr">
         <is>
-          <t>277810</t>
+          <t>041190</t>
         </is>
       </c>
       <c r="D38" s="16" t="inlineStr">
         <is>
-          <t>레인보우로보틱스</t>
+          <t>우리기술투자</t>
         </is>
       </c>
       <c r="E38" s="17" t="n">
-        <v>7211</v>
+        <v>5517</v>
       </c>
       <c r="F38" s="18" t="n">
         <v>1</v>
@@ -1511,23 +1511,23 @@
     </row>
     <row r="39">
       <c r="A39" s="14" t="n">
-        <v>44515</v>
+        <v>45849</v>
       </c>
       <c r="B39" s="14" t="n">
-        <v>45923</v>
+        <v>45926</v>
       </c>
       <c r="C39" s="15" t="inlineStr">
         <is>
-          <t>068270</t>
+          <t>060250</t>
         </is>
       </c>
       <c r="D39" s="16" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>NHN KCP</t>
         </is>
       </c>
       <c r="E39" s="17" t="n">
-        <v>5000</v>
+        <v>9171</v>
       </c>
       <c r="F39" s="18" t="n">
         <v>1</v>
@@ -1535,23 +1535,23 @@
     </row>
     <row r="40">
       <c r="A40" s="14" t="n">
-        <v>45922</v>
+        <v>45925</v>
       </c>
       <c r="B40" s="14" t="n">
-        <v>45923</v>
+        <v>45925</v>
       </c>
       <c r="C40" s="15" t="inlineStr">
         <is>
-          <t>347850</t>
+          <t>277810</t>
         </is>
       </c>
       <c r="D40" s="16" t="inlineStr">
         <is>
-          <t>디앤디파마텍</t>
+          <t>레인보우로보틱스</t>
         </is>
       </c>
       <c r="E40" s="17" t="n">
-        <v>5000</v>
+        <v>7211</v>
       </c>
       <c r="F40" s="18" t="n">
         <v>1</v>
@@ -1559,19 +1559,19 @@
     </row>
     <row r="41">
       <c r="A41" s="14" t="n">
-        <v>45377</v>
+        <v>44515</v>
       </c>
       <c r="B41" s="14" t="n">
-        <v>45919</v>
+        <v>45923</v>
       </c>
       <c r="C41" s="15" t="inlineStr">
         <is>
-          <t>000250</t>
+          <t>068270</t>
         </is>
       </c>
       <c r="D41" s="16" t="inlineStr">
         <is>
-          <t>삼천당제약</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="E41" s="17" t="n">
@@ -1583,19 +1583,19 @@
     </row>
     <row r="42">
       <c r="A42" s="14" t="n">
-        <v>45839</v>
+        <v>45922</v>
       </c>
       <c r="B42" s="14" t="n">
-        <v>45919</v>
+        <v>45923</v>
       </c>
       <c r="C42" s="15" t="inlineStr">
         <is>
-          <t>064260</t>
+          <t>347850</t>
         </is>
       </c>
       <c r="D42" s="16" t="inlineStr">
         <is>
-          <t>다날</t>
+          <t>디앤디파마텍</t>
         </is>
       </c>
       <c r="E42" s="17" t="n">
@@ -1607,19 +1607,19 @@
     </row>
     <row r="43">
       <c r="A43" s="14" t="n">
-        <v>45918</v>
+        <v>45377</v>
       </c>
       <c r="B43" s="14" t="n">
         <v>45919</v>
       </c>
       <c r="C43" s="15" t="inlineStr">
         <is>
-          <t>090360</t>
+          <t>000250</t>
         </is>
       </c>
       <c r="D43" s="16" t="inlineStr">
         <is>
-          <t>로보스타</t>
+          <t>삼천당제약</t>
         </is>
       </c>
       <c r="E43" s="17" t="n">
@@ -1631,19 +1631,19 @@
     </row>
     <row r="44">
       <c r="A44" s="14" t="n">
-        <v>45708</v>
+        <v>45839</v>
       </c>
       <c r="B44" s="14" t="n">
         <v>45919</v>
       </c>
       <c r="C44" s="15" t="inlineStr">
         <is>
-          <t>047810</t>
+          <t>064260</t>
         </is>
       </c>
       <c r="D44" s="16" t="inlineStr">
         <is>
-          <t>한국항공우주</t>
+          <t>다날</t>
         </is>
       </c>
       <c r="E44" s="17" t="n">
@@ -1655,19 +1655,19 @@
     </row>
     <row r="45">
       <c r="A45" s="14" t="n">
-        <v>45883</v>
+        <v>45918</v>
       </c>
       <c r="B45" s="14" t="n">
-        <v>45912</v>
+        <v>45919</v>
       </c>
       <c r="C45" s="15" t="inlineStr">
         <is>
-          <t>456160</t>
+          <t>090360</t>
         </is>
       </c>
       <c r="D45" s="16" t="inlineStr">
         <is>
-          <t>지투지바이오</t>
+          <t>로보스타</t>
         </is>
       </c>
       <c r="E45" s="17" t="n">
@@ -1679,19 +1679,19 @@
     </row>
     <row r="46">
       <c r="A46" s="14" t="n">
-        <v>45912</v>
+        <v>45708</v>
       </c>
       <c r="B46" s="14" t="n">
-        <v>45912</v>
+        <v>45919</v>
       </c>
       <c r="C46" s="15" t="inlineStr">
         <is>
-          <t>004370</t>
+          <t>047810</t>
         </is>
       </c>
       <c r="D46" s="16" t="inlineStr">
         <is>
-          <t>농심</t>
+          <t>한국항공우주</t>
         </is>
       </c>
       <c r="E46" s="17" t="n">
@@ -1703,19 +1703,19 @@
     </row>
     <row r="47">
       <c r="A47" s="14" t="n">
-        <v>45911</v>
+        <v>45883</v>
       </c>
       <c r="B47" s="14" t="n">
         <v>45912</v>
       </c>
       <c r="C47" s="15" t="inlineStr">
         <is>
-          <t>100090</t>
+          <t>456160</t>
         </is>
       </c>
       <c r="D47" s="16" t="inlineStr">
         <is>
-          <t>SK오션플랜트</t>
+          <t>지투지바이오</t>
         </is>
       </c>
       <c r="E47" s="17" t="n">
@@ -1727,19 +1727,19 @@
     </row>
     <row r="48">
       <c r="A48" s="14" t="n">
-        <v>45908</v>
+        <v>45912</v>
       </c>
       <c r="B48" s="14" t="n">
-        <v>45910</v>
+        <v>45912</v>
       </c>
       <c r="C48" s="15" t="inlineStr">
         <is>
-          <t>075580</t>
+          <t>004370</t>
         </is>
       </c>
       <c r="D48" s="16" t="inlineStr">
         <is>
-          <t>세진중공업</t>
+          <t>농심</t>
         </is>
       </c>
       <c r="E48" s="17" t="n">
@@ -1751,19 +1751,19 @@
     </row>
     <row r="49">
       <c r="A49" s="14" t="n">
-        <v>45908</v>
+        <v>45911</v>
       </c>
       <c r="B49" s="14" t="n">
-        <v>45908</v>
+        <v>45912</v>
       </c>
       <c r="C49" s="15" t="inlineStr">
         <is>
-          <t>290650</t>
+          <t>100090</t>
         </is>
       </c>
       <c r="D49" s="16" t="inlineStr">
         <is>
-          <t>엘앤씨바이오</t>
+          <t>SK오션플랜트</t>
         </is>
       </c>
       <c r="E49" s="17" t="n">
@@ -1775,19 +1775,19 @@
     </row>
     <row r="50">
       <c r="A50" s="14" t="n">
-        <v>45898</v>
+        <v>45908</v>
       </c>
       <c r="B50" s="14" t="n">
-        <v>45898</v>
+        <v>45910</v>
       </c>
       <c r="C50" s="15" t="inlineStr">
         <is>
-          <t>082740</t>
+          <t>075580</t>
         </is>
       </c>
       <c r="D50" s="16" t="inlineStr">
         <is>
-          <t>한화엔진</t>
+          <t>세진중공업</t>
         </is>
       </c>
       <c r="E50" s="17" t="n">
@@ -1799,19 +1799,19 @@
     </row>
     <row r="51">
       <c r="A51" s="14" t="n">
-        <v>45897</v>
+        <v>45908</v>
       </c>
       <c r="B51" s="14" t="n">
-        <v>45897</v>
+        <v>45908</v>
       </c>
       <c r="C51" s="15" t="inlineStr">
         <is>
-          <t>460930</t>
+          <t>290650</t>
         </is>
       </c>
       <c r="D51" s="16" t="inlineStr">
         <is>
-          <t>현대힘스</t>
+          <t>엘앤씨바이오</t>
         </is>
       </c>
       <c r="E51" s="17" t="n">
@@ -1823,19 +1823,19 @@
     </row>
     <row r="52">
       <c r="A52" s="14" t="n">
-        <v>45897</v>
+        <v>45898</v>
       </c>
       <c r="B52" s="14" t="n">
-        <v>45897</v>
+        <v>45898</v>
       </c>
       <c r="C52" s="15" t="inlineStr">
         <is>
-          <t>009540</t>
+          <t>082740</t>
         </is>
       </c>
       <c r="D52" s="16" t="inlineStr">
         <is>
-          <t>HD한국조선해양</t>
+          <t>한화엔진</t>
         </is>
       </c>
       <c r="E52" s="17" t="n">
@@ -1847,19 +1847,19 @@
     </row>
     <row r="53">
       <c r="A53" s="14" t="n">
-        <v>45896</v>
+        <v>45897</v>
       </c>
       <c r="B53" s="14" t="n">
         <v>45897</v>
       </c>
       <c r="C53" s="15" t="inlineStr">
         <is>
-          <t>010620</t>
+          <t>460930</t>
         </is>
       </c>
       <c r="D53" s="16" t="inlineStr">
         <is>
-          <t>HD현대미포</t>
+          <t>현대힘스</t>
         </is>
       </c>
       <c r="E53" s="17" t="n">
@@ -1871,19 +1871,19 @@
     </row>
     <row r="54">
       <c r="A54" s="14" t="n">
-        <v>45895</v>
+        <v>45897</v>
       </c>
       <c r="B54" s="14" t="n">
-        <v>45895</v>
+        <v>45897</v>
       </c>
       <c r="C54" s="15" t="inlineStr">
         <is>
-          <t>298040</t>
+          <t>009540</t>
         </is>
       </c>
       <c r="D54" s="16" t="inlineStr">
         <is>
-          <t>효성중공업</t>
+          <t>HD한국조선해양</t>
         </is>
       </c>
       <c r="E54" s="17" t="n">
@@ -1895,19 +1895,19 @@
     </row>
     <row r="55">
       <c r="A55" s="14" t="n">
-        <v>45782</v>
+        <v>45896</v>
       </c>
       <c r="B55" s="14" t="n">
-        <v>45895</v>
+        <v>45897</v>
       </c>
       <c r="C55" s="15" t="inlineStr">
         <is>
-          <t>079550</t>
+          <t>010620</t>
         </is>
       </c>
       <c r="D55" s="16" t="inlineStr">
         <is>
-          <t>LIG넥스원</t>
+          <t>HD현대미포</t>
         </is>
       </c>
       <c r="E55" s="17" t="n">
@@ -1919,19 +1919,19 @@
     </row>
     <row r="56">
       <c r="A56" s="14" t="n">
-        <v>45888</v>
+        <v>45895</v>
       </c>
       <c r="B56" s="14" t="n">
-        <v>45888</v>
+        <v>45895</v>
       </c>
       <c r="C56" s="15" t="inlineStr">
         <is>
-          <t>0008Z0</t>
+          <t>298040</t>
         </is>
       </c>
       <c r="D56" s="16" t="inlineStr">
         <is>
-          <t>에스엔시스</t>
+          <t>효성중공업</t>
         </is>
       </c>
       <c r="E56" s="17" t="n">
@@ -1943,19 +1943,19 @@
     </row>
     <row r="57">
       <c r="A57" s="14" t="n">
-        <v>45887</v>
+        <v>45782</v>
       </c>
       <c r="B57" s="14" t="n">
-        <v>45887</v>
+        <v>45895</v>
       </c>
       <c r="C57" s="15" t="inlineStr">
         <is>
-          <t>484590</t>
+          <t>079550</t>
         </is>
       </c>
       <c r="D57" s="16" t="inlineStr">
         <is>
-          <t>삼양컴텍</t>
+          <t>LIG넥스원</t>
         </is>
       </c>
       <c r="E57" s="17" t="n">
@@ -1967,19 +1967,19 @@
     </row>
     <row r="58">
       <c r="A58" s="14" t="n">
-        <v>45755</v>
+        <v>45888</v>
       </c>
       <c r="B58" s="14" t="n">
-        <v>45883</v>
+        <v>45888</v>
       </c>
       <c r="C58" s="15" t="inlineStr">
         <is>
-          <t>298380</t>
+          <t>0008Z0</t>
         </is>
       </c>
       <c r="D58" s="16" t="inlineStr">
         <is>
-          <t>에이비엘바이오</t>
+          <t>에스엔시스</t>
         </is>
       </c>
       <c r="E58" s="17" t="n">
@@ -1991,19 +1991,19 @@
     </row>
     <row r="59">
       <c r="A59" s="14" t="n">
-        <v>45882</v>
+        <v>45887</v>
       </c>
       <c r="B59" s="14" t="n">
-        <v>45882</v>
+        <v>45887</v>
       </c>
       <c r="C59" s="15" t="inlineStr">
         <is>
-          <t>034220</t>
+          <t>484590</t>
         </is>
       </c>
       <c r="D59" s="16" t="inlineStr">
         <is>
-          <t>LG디스플레이</t>
+          <t>삼양컴텍</t>
         </is>
       </c>
       <c r="E59" s="17" t="n">
@@ -2015,19 +2015,19 @@
     </row>
     <row r="60">
       <c r="A60" s="14" t="n">
-        <v>45870</v>
+        <v>45755</v>
       </c>
       <c r="B60" s="14" t="n">
-        <v>45876</v>
+        <v>45883</v>
       </c>
       <c r="C60" s="15" t="inlineStr">
         <is>
-          <t>439260</t>
+          <t>298380</t>
         </is>
       </c>
       <c r="D60" s="16" t="inlineStr">
         <is>
-          <t>대한조선</t>
+          <t>에이비엘바이오</t>
         </is>
       </c>
       <c r="E60" s="17" t="n">
@@ -2039,19 +2039,19 @@
     </row>
     <row r="61">
       <c r="A61" s="14" t="n">
-        <v>45785</v>
+        <v>45882</v>
       </c>
       <c r="B61" s="14" t="n">
-        <v>45875</v>
+        <v>45882</v>
       </c>
       <c r="C61" s="15" t="inlineStr">
         <is>
-          <t>278470</t>
+          <t>034220</t>
         </is>
       </c>
       <c r="D61" s="16" t="inlineStr">
         <is>
-          <t>에이피알</t>
+          <t>LG디스플레이</t>
         </is>
       </c>
       <c r="E61" s="17" t="n">
@@ -2063,19 +2063,19 @@
     </row>
     <row r="62">
       <c r="A62" s="14" t="n">
-        <v>45874</v>
+        <v>45870</v>
       </c>
       <c r="B62" s="14" t="n">
-        <v>45874</v>
+        <v>45876</v>
       </c>
       <c r="C62" s="15" t="inlineStr">
         <is>
-          <t>326030</t>
+          <t>439260</t>
         </is>
       </c>
       <c r="D62" s="16" t="inlineStr">
         <is>
-          <t>SK바이오팜</t>
+          <t>대한조선</t>
         </is>
       </c>
       <c r="E62" s="17" t="n">
@@ -2087,19 +2087,19 @@
     </row>
     <row r="63">
       <c r="A63" s="14" t="n">
-        <v>45699</v>
+        <v>45785</v>
       </c>
       <c r="B63" s="14" t="n">
-        <v>45870</v>
+        <v>45875</v>
       </c>
       <c r="C63" s="15" t="inlineStr">
         <is>
-          <t>012450</t>
+          <t>278470</t>
         </is>
       </c>
       <c r="D63" s="16" t="inlineStr">
         <is>
-          <t>한화에어로스페이스</t>
+          <t>에이피알</t>
         </is>
       </c>
       <c r="E63" s="17" t="n">
@@ -2111,19 +2111,19 @@
     </row>
     <row r="64">
       <c r="A64" s="14" t="n">
-        <v>45700</v>
+        <v>45874</v>
       </c>
       <c r="B64" s="14" t="n">
-        <v>45869</v>
+        <v>45874</v>
       </c>
       <c r="C64" s="15" t="inlineStr">
         <is>
-          <t>272210</t>
+          <t>326030</t>
         </is>
       </c>
       <c r="D64" s="16" t="inlineStr">
         <is>
-          <t>한화시스템</t>
+          <t>SK바이오팜</t>
         </is>
       </c>
       <c r="E64" s="17" t="n">
@@ -2135,19 +2135,19 @@
     </row>
     <row r="65">
       <c r="A65" s="14" t="n">
-        <v>45772</v>
+        <v>45699</v>
       </c>
       <c r="B65" s="14" t="n">
-        <v>45868</v>
+        <v>45870</v>
       </c>
       <c r="C65" s="15" t="inlineStr">
         <is>
-          <t>009830</t>
+          <t>012450</t>
         </is>
       </c>
       <c r="D65" s="16" t="inlineStr">
         <is>
-          <t>한화솔루션</t>
+          <t>한화에어로스페이스</t>
         </is>
       </c>
       <c r="E65" s="17" t="n">
@@ -2159,19 +2159,19 @@
     </row>
     <row r="66">
       <c r="A66" s="14" t="n">
-        <v>45868</v>
+        <v>45772</v>
       </c>
       <c r="B66" s="14" t="n">
         <v>45868</v>
       </c>
       <c r="C66" s="15" t="inlineStr">
         <is>
-          <t>009150</t>
+          <t>009830</t>
         </is>
       </c>
       <c r="D66" s="16" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>한화솔루션</t>
         </is>
       </c>
       <c r="E66" s="17" t="n">
@@ -2183,19 +2183,19 @@
     </row>
     <row r="67">
       <c r="A67" s="14" t="n">
-        <v>45867</v>
+        <v>45868</v>
       </c>
       <c r="B67" s="14" t="n">
-        <v>45867</v>
+        <v>45868</v>
       </c>
       <c r="C67" s="15" t="inlineStr">
         <is>
-          <t>489790</t>
+          <t>009150</t>
         </is>
       </c>
       <c r="D67" s="16" t="inlineStr">
         <is>
-          <t>한화비전</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="E67" s="17" t="n">
@@ -2207,19 +2207,19 @@
     </row>
     <row r="68">
       <c r="A68" s="14" t="n">
-        <v>45862</v>
+        <v>45867</v>
       </c>
       <c r="B68" s="14" t="n">
         <v>45867</v>
       </c>
       <c r="C68" s="15" t="inlineStr">
         <is>
-          <t>042670</t>
+          <t>489790</t>
         </is>
       </c>
       <c r="D68" s="16" t="inlineStr">
         <is>
-          <t>HD현대인프라코어</t>
+          <t>한화비전</t>
         </is>
       </c>
       <c r="E68" s="17" t="n">
@@ -2231,19 +2231,19 @@
     </row>
     <row r="69">
       <c r="A69" s="14" t="n">
-        <v>45861</v>
+        <v>45862</v>
       </c>
       <c r="B69" s="14" t="n">
-        <v>45861</v>
+        <v>45867</v>
       </c>
       <c r="C69" s="15" t="inlineStr">
         <is>
-          <t>484120</t>
+          <t>042670</t>
         </is>
       </c>
       <c r="D69" s="16" t="inlineStr">
         <is>
-          <t>도우인시스</t>
+          <t>HD현대인프라코어</t>
         </is>
       </c>
       <c r="E69" s="17" t="n">
@@ -2255,19 +2255,19 @@
     </row>
     <row r="70">
       <c r="A70" s="14" t="n">
-        <v>45846</v>
+        <v>45861</v>
       </c>
       <c r="B70" s="14" t="n">
         <v>45861</v>
       </c>
       <c r="C70" s="15" t="inlineStr">
         <is>
-          <t>008970</t>
+          <t>484120</t>
         </is>
       </c>
       <c r="D70" s="16" t="inlineStr">
         <is>
-          <t>KBI동양철관</t>
+          <t>도우인시스</t>
         </is>
       </c>
       <c r="E70" s="17" t="n">
@@ -2279,19 +2279,19 @@
     </row>
     <row r="71">
       <c r="A71" s="14" t="n">
-        <v>45860</v>
+        <v>45846</v>
       </c>
       <c r="B71" s="14" t="n">
-        <v>45860</v>
+        <v>45861</v>
       </c>
       <c r="C71" s="15" t="inlineStr">
         <is>
-          <t>037270</t>
+          <t>008970</t>
         </is>
       </c>
       <c r="D71" s="16" t="inlineStr">
         <is>
-          <t>YG PLUS</t>
+          <t>KBI동양철관</t>
         </is>
       </c>
       <c r="E71" s="17" t="n">
@@ -2303,19 +2303,19 @@
     </row>
     <row r="72">
       <c r="A72" s="14" t="n">
-        <v>45856</v>
+        <v>45860</v>
       </c>
       <c r="B72" s="14" t="n">
-        <v>45856</v>
+        <v>45860</v>
       </c>
       <c r="C72" s="15" t="inlineStr">
         <is>
-          <t>141080</t>
+          <t>037270</t>
         </is>
       </c>
       <c r="D72" s="16" t="inlineStr">
         <is>
-          <t>리가켐바이오</t>
+          <t>YG PLUS</t>
         </is>
       </c>
       <c r="E72" s="17" t="n">
@@ -2327,19 +2327,19 @@
     </row>
     <row r="73">
       <c r="A73" s="14" t="n">
-        <v>45854</v>
+        <v>45856</v>
       </c>
       <c r="B73" s="14" t="n">
-        <v>45854</v>
+        <v>45856</v>
       </c>
       <c r="C73" s="15" t="inlineStr">
         <is>
-          <t>294570</t>
+          <t>141080</t>
         </is>
       </c>
       <c r="D73" s="16" t="inlineStr">
         <is>
-          <t>쿠콘</t>
+          <t>리가켐바이오</t>
         </is>
       </c>
       <c r="E73" s="17" t="n">
@@ -2358,12 +2358,12 @@
       </c>
       <c r="C74" s="15" t="inlineStr">
         <is>
-          <t>441270</t>
+          <t>294570</t>
         </is>
       </c>
       <c r="D74" s="16" t="inlineStr">
         <is>
-          <t>파인엠텍</t>
+          <t>쿠콘</t>
         </is>
       </c>
       <c r="E74" s="17" t="n">
@@ -2375,19 +2375,19 @@
     </row>
     <row r="75">
       <c r="A75" s="14" t="n">
-        <v>45849</v>
+        <v>45854</v>
       </c>
       <c r="B75" s="14" t="n">
-        <v>45849</v>
+        <v>45854</v>
       </c>
       <c r="C75" s="15" t="inlineStr">
         <is>
-          <t>402340</t>
+          <t>441270</t>
         </is>
       </c>
       <c r="D75" s="16" t="inlineStr">
         <is>
-          <t>SK스퀘어</t>
+          <t>파인엠텍</t>
         </is>
       </c>
       <c r="E75" s="17" t="n">
@@ -2399,19 +2399,19 @@
     </row>
     <row r="76">
       <c r="A76" s="14" t="n">
-        <v>45841</v>
+        <v>45849</v>
       </c>
       <c r="B76" s="14" t="n">
-        <v>45842</v>
+        <v>45849</v>
       </c>
       <c r="C76" s="15" t="inlineStr">
         <is>
-          <t>005490</t>
+          <t>402340</t>
         </is>
       </c>
       <c r="D76" s="16" t="inlineStr">
         <is>
-          <t>POSCO홀딩스</t>
+          <t>SK스퀘어</t>
         </is>
       </c>
       <c r="E76" s="17" t="n">
@@ -2423,19 +2423,19 @@
     </row>
     <row r="77">
       <c r="A77" s="14" t="n">
-        <v>45840</v>
+        <v>45841</v>
       </c>
       <c r="B77" s="14" t="n">
-        <v>45840</v>
+        <v>45842</v>
       </c>
       <c r="C77" s="15" t="inlineStr">
         <is>
-          <t>267270</t>
+          <t>005490</t>
         </is>
       </c>
       <c r="D77" s="16" t="inlineStr">
         <is>
-          <t>HD현대건설기계</t>
+          <t>POSCO홀딩스</t>
         </is>
       </c>
       <c r="E77" s="17" t="n">
@@ -2447,19 +2447,19 @@
     </row>
     <row r="78">
       <c r="A78" s="14" t="n">
-        <v>45839</v>
+        <v>45840</v>
       </c>
       <c r="B78" s="14" t="n">
-        <v>45839</v>
+        <v>45840</v>
       </c>
       <c r="C78" s="15" t="inlineStr">
         <is>
-          <t>000880</t>
+          <t>267270</t>
         </is>
       </c>
       <c r="D78" s="16" t="inlineStr">
         <is>
-          <t>한화</t>
+          <t>HD현대건설기계</t>
         </is>
       </c>
       <c r="E78" s="17" t="n">
@@ -2471,19 +2471,19 @@
     </row>
     <row r="79">
       <c r="A79" s="14" t="n">
-        <v>43997</v>
+        <v>45839</v>
       </c>
       <c r="B79" s="14" t="n">
         <v>45839</v>
       </c>
       <c r="C79" s="15" t="inlineStr">
         <is>
-          <t>034730</t>
+          <t>000880</t>
         </is>
       </c>
       <c r="D79" s="16" t="inlineStr">
         <is>
-          <t>SK</t>
+          <t>한화</t>
         </is>
       </c>
       <c r="E79" s="17" t="n">
@@ -2495,25 +2495,49 @@
     </row>
     <row r="80">
       <c r="A80" s="14" t="n">
-        <v>45838</v>
+        <v>43997</v>
       </c>
       <c r="B80" s="14" t="n">
         <v>45839</v>
       </c>
       <c r="C80" s="15" t="inlineStr">
         <is>
+          <t>034730</t>
+        </is>
+      </c>
+      <c r="D80" s="16" t="inlineStr">
+        <is>
+          <t>SK</t>
+        </is>
+      </c>
+      <c r="E80" s="17" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F80" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="14" t="n">
+        <v>45838</v>
+      </c>
+      <c r="B81" s="14" t="n">
+        <v>45839</v>
+      </c>
+      <c r="C81" s="15" t="inlineStr">
+        <is>
           <t>096770</t>
         </is>
       </c>
-      <c r="D80" s="16" t="inlineStr">
+      <c r="D81" s="16" t="inlineStr">
         <is>
           <t>SK이노베이션</t>
         </is>
       </c>
-      <c r="E80" s="17" t="n">
-        <v>5000</v>
-      </c>
-      <c r="F80" s="18" t="n">
+      <c r="E81" s="17" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F81" s="18" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update S12 system: monitor improvements, scheduler setup, and documentation
</commit_message>
<xml_diff>
--- a/output/turnover_universe.xlsx
+++ b/output/turnover_universe.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12180" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="universe" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="universe" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -573,7 +573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H81"/>
+  <dimension ref="A1:H82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -617,7 +617,7 @@
       </c>
       <c r="H1" s="13" t="inlineStr">
         <is>
-          <t>최종 업데이트: 2025-10-30</t>
+          <t>최종 업데이트: 2025-11-02</t>
         </is>
       </c>
     </row>
@@ -626,7 +626,7 @@
         <v>45942</v>
       </c>
       <c r="B2" s="14" t="n">
-        <v>45960</v>
+        <v>45963</v>
       </c>
       <c r="C2" s="15" t="inlineStr">
         <is>
@@ -639,10 +639,10 @@
         </is>
       </c>
       <c r="E2" s="17" t="n">
-        <v>61144.41</v>
+        <v>83542.09</v>
       </c>
       <c r="F2" s="18" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3">
@@ -650,7 +650,7 @@
         <v>45942</v>
       </c>
       <c r="B3" s="14" t="n">
-        <v>45960</v>
+        <v>45963</v>
       </c>
       <c r="C3" s="15" t="inlineStr">
         <is>
@@ -663,10 +663,10 @@
         </is>
       </c>
       <c r="E3" s="17" t="n">
-        <v>48948.26</v>
+        <v>30699.54</v>
       </c>
       <c r="F3" s="18" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4">
@@ -674,7 +674,7 @@
         <v>45942</v>
       </c>
       <c r="B4" s="14" t="n">
-        <v>45960</v>
+        <v>45963</v>
       </c>
       <c r="C4" s="15" t="inlineStr">
         <is>
@@ -687,10 +687,10 @@
         </is>
       </c>
       <c r="E4" s="17" t="n">
-        <v>21336.9</v>
+        <v>10173.87</v>
       </c>
       <c r="F4" s="18" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5">
@@ -698,7 +698,7 @@
         <v>45604</v>
       </c>
       <c r="B5" s="14" t="n">
-        <v>45960</v>
+        <v>45963</v>
       </c>
       <c r="C5" s="15" t="inlineStr">
         <is>
@@ -711,10 +711,10 @@
         </is>
       </c>
       <c r="E5" s="17" t="n">
-        <v>24575.94</v>
+        <v>5344.56</v>
       </c>
       <c r="F5" s="18" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6">
@@ -722,7 +722,7 @@
         <v>45942</v>
       </c>
       <c r="B6" s="14" t="n">
-        <v>45960</v>
+        <v>45963</v>
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
@@ -735,10 +735,10 @@
         </is>
       </c>
       <c r="E6" s="17" t="n">
-        <v>7437.190000000001</v>
+        <v>15661.46</v>
       </c>
       <c r="F6" s="18" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7">
@@ -746,7 +746,7 @@
         <v>45730</v>
       </c>
       <c r="B7" s="14" t="n">
-        <v>45960</v>
+        <v>45963</v>
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
@@ -759,31 +759,31 @@
         </is>
       </c>
       <c r="E7" s="17" t="n">
-        <v>10935.75</v>
+        <v>5928.5</v>
       </c>
       <c r="F7" s="18" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>45942</v>
+        <v>45833</v>
       </c>
       <c r="B8" s="14" t="n">
-        <v>45960</v>
+        <v>45963</v>
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>042700</t>
+          <t>005380</t>
         </is>
       </c>
       <c r="D8" s="16" t="inlineStr">
         <is>
-          <t>한미반도체</t>
+          <t>현대차</t>
         </is>
       </c>
       <c r="E8" s="17" t="n">
-        <v>6500.89</v>
+        <v>22349.1</v>
       </c>
       <c r="F8" s="18" t="n">
         <v>8</v>
@@ -791,26 +791,26 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>45833</v>
+        <v>45942</v>
       </c>
       <c r="B9" s="14" t="n">
         <v>45960</v>
       </c>
       <c r="C9" s="15" t="inlineStr">
         <is>
-          <t>005380</t>
+          <t>042700</t>
         </is>
       </c>
       <c r="D9" s="16" t="inlineStr">
         <is>
-          <t>현대차</t>
+          <t>한미반도체</t>
         </is>
       </c>
       <c r="E9" s="17" t="n">
-        <v>18592.32</v>
+        <v>6500.89</v>
       </c>
       <c r="F9" s="18" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10">
@@ -959,23 +959,23 @@
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
-        <v>45947</v>
+        <v>45942</v>
       </c>
       <c r="B16" s="14" t="n">
-        <v>45960</v>
+        <v>45963</v>
       </c>
       <c r="C16" s="15" t="inlineStr">
         <is>
-          <t>066970</t>
+          <t>005935</t>
         </is>
       </c>
       <c r="D16" s="16" t="inlineStr">
         <is>
-          <t>엘앤에프</t>
+          <t>삼성전자우</t>
         </is>
       </c>
       <c r="E16" s="17" t="n">
-        <v>5207</v>
+        <v>5133.84</v>
       </c>
       <c r="F16" s="18" t="n">
         <v>3</v>
@@ -986,20 +986,20 @@
         <v>45947</v>
       </c>
       <c r="B17" s="14" t="n">
-        <v>45952</v>
+        <v>45960</v>
       </c>
       <c r="C17" s="15" t="inlineStr">
         <is>
-          <t>051910</t>
+          <t>066970</t>
         </is>
       </c>
       <c r="D17" s="16" t="inlineStr">
         <is>
-          <t>LG화학</t>
+          <t>엘앤에프</t>
         </is>
       </c>
       <c r="E17" s="17" t="n">
-        <v>9404.630000000001</v>
+        <v>5207</v>
       </c>
       <c r="F17" s="18" t="n">
         <v>3</v>
@@ -1010,20 +1010,20 @@
         <v>45947</v>
       </c>
       <c r="B18" s="14" t="n">
-        <v>45949</v>
+        <v>45952</v>
       </c>
       <c r="C18" s="15" t="inlineStr">
         <is>
-          <t>450080</t>
+          <t>051910</t>
         </is>
       </c>
       <c r="D18" s="16" t="inlineStr">
         <is>
-          <t>에코프로머티</t>
+          <t>LG화학</t>
         </is>
       </c>
       <c r="E18" s="17" t="n">
-        <v>7222.29</v>
+        <v>9404.630000000001</v>
       </c>
       <c r="F18" s="18" t="n">
         <v>3</v>
@@ -1031,23 +1031,23 @@
     </row>
     <row r="19">
       <c r="A19" s="14" t="n">
-        <v>45853</v>
+        <v>45947</v>
       </c>
       <c r="B19" s="14" t="n">
         <v>45949</v>
       </c>
       <c r="C19" s="15" t="inlineStr">
         <is>
-          <t>015760</t>
+          <t>450080</t>
         </is>
       </c>
       <c r="D19" s="16" t="inlineStr">
         <is>
-          <t>한국전력</t>
+          <t>에코프로머티</t>
         </is>
       </c>
       <c r="E19" s="17" t="n">
-        <v>6619.35</v>
+        <v>7222.29</v>
       </c>
       <c r="F19" s="18" t="n">
         <v>3</v>
@@ -1055,47 +1055,47 @@
     </row>
     <row r="20">
       <c r="A20" s="14" t="n">
-        <v>45942</v>
+        <v>45853</v>
       </c>
       <c r="B20" s="14" t="n">
-        <v>45960</v>
+        <v>45949</v>
       </c>
       <c r="C20" s="15" t="inlineStr">
         <is>
-          <t>108490</t>
+          <t>015760</t>
         </is>
       </c>
       <c r="D20" s="16" t="inlineStr">
         <is>
-          <t>로보티즈</t>
+          <t>한국전력</t>
         </is>
       </c>
       <c r="E20" s="17" t="n">
-        <v>6265.45</v>
+        <v>6619.35</v>
       </c>
       <c r="F20" s="18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="14" t="n">
-        <v>45942</v>
+        <v>45960</v>
       </c>
       <c r="B21" s="14" t="n">
-        <v>45960</v>
+        <v>45963</v>
       </c>
       <c r="C21" s="15" t="inlineStr">
         <is>
-          <t>005935</t>
+          <t>000270</t>
         </is>
       </c>
       <c r="D21" s="16" t="inlineStr">
         <is>
-          <t>삼성전자우</t>
+          <t>기아</t>
         </is>
       </c>
       <c r="E21" s="17" t="n">
-        <v>6234.82</v>
+        <v>5542.92</v>
       </c>
       <c r="F21" s="18" t="n">
         <v>2</v>
@@ -1103,23 +1103,23 @@
     </row>
     <row r="22">
       <c r="A22" s="14" t="n">
-        <v>45700</v>
+        <v>45959</v>
       </c>
       <c r="B22" s="14" t="n">
-        <v>45960</v>
+        <v>45963</v>
       </c>
       <c r="C22" s="15" t="inlineStr">
         <is>
-          <t>272210</t>
+          <t>001440</t>
         </is>
       </c>
       <c r="D22" s="16" t="inlineStr">
         <is>
-          <t>한화시스템</t>
+          <t>대한전선</t>
         </is>
       </c>
       <c r="E22" s="17" t="n">
-        <v>14791.78</v>
+        <v>9763.82</v>
       </c>
       <c r="F22" s="18" t="n">
         <v>2</v>
@@ -1127,23 +1127,23 @@
     </row>
     <row r="23">
       <c r="A23" s="14" t="n">
-        <v>45958</v>
+        <v>45925</v>
       </c>
       <c r="B23" s="14" t="n">
-        <v>45959</v>
+        <v>45963</v>
       </c>
       <c r="C23" s="15" t="inlineStr">
         <is>
-          <t>336260</t>
+          <t>277810</t>
         </is>
       </c>
       <c r="D23" s="16" t="inlineStr">
         <is>
-          <t>두산퓨얼셀</t>
+          <t>레인보우로보틱스</t>
         </is>
       </c>
       <c r="E23" s="17" t="n">
-        <v>5907.51</v>
+        <v>20078.78</v>
       </c>
       <c r="F23" s="18" t="n">
         <v>2</v>
@@ -1151,23 +1151,23 @@
     </row>
     <row r="24">
       <c r="A24" s="14" t="n">
-        <v>45957</v>
+        <v>45922</v>
       </c>
       <c r="B24" s="14" t="n">
-        <v>45959</v>
+        <v>45963</v>
       </c>
       <c r="C24" s="15" t="inlineStr">
         <is>
-          <t>000720</t>
+          <t>347850</t>
         </is>
       </c>
       <c r="D24" s="16" t="inlineStr">
         <is>
-          <t>현대건설</t>
+          <t>디앤디파마텍</t>
         </is>
       </c>
       <c r="E24" s="17" t="n">
-        <v>7859.2</v>
+        <v>5363.72</v>
       </c>
       <c r="F24" s="18" t="n">
         <v>2</v>
@@ -1175,23 +1175,23 @@
     </row>
     <row r="25">
       <c r="A25" s="14" t="n">
-        <v>45650</v>
+        <v>45942</v>
       </c>
       <c r="B25" s="14" t="n">
-        <v>45957</v>
+        <v>45960</v>
       </c>
       <c r="C25" s="15" t="inlineStr">
         <is>
-          <t>196170</t>
+          <t>108490</t>
         </is>
       </c>
       <c r="D25" s="16" t="inlineStr">
         <is>
-          <t>알테오젠</t>
+          <t>로보티즈</t>
         </is>
       </c>
       <c r="E25" s="17" t="n">
-        <v>6894.2</v>
+        <v>6265.45</v>
       </c>
       <c r="F25" s="18" t="n">
         <v>2</v>
@@ -1199,23 +1199,23 @@
     </row>
     <row r="26">
       <c r="A26" s="14" t="n">
-        <v>45876</v>
+        <v>45700</v>
       </c>
       <c r="B26" s="14" t="n">
-        <v>45957</v>
+        <v>45960</v>
       </c>
       <c r="C26" s="15" t="inlineStr">
         <is>
-          <t>097230</t>
+          <t>272210</t>
         </is>
       </c>
       <c r="D26" s="16" t="inlineStr">
         <is>
-          <t>HJ중공업</t>
+          <t>한화시스템</t>
         </is>
       </c>
       <c r="E26" s="17" t="n">
-        <v>6016.41</v>
+        <v>14791.78</v>
       </c>
       <c r="F26" s="18" t="n">
         <v>2</v>
@@ -1223,23 +1223,23 @@
     </row>
     <row r="27">
       <c r="A27" s="14" t="n">
-        <v>45694</v>
+        <v>45958</v>
       </c>
       <c r="B27" s="14" t="n">
-        <v>45952</v>
+        <v>45959</v>
       </c>
       <c r="C27" s="15" t="inlineStr">
         <is>
-          <t>064350</t>
+          <t>336260</t>
         </is>
       </c>
       <c r="D27" s="16" t="inlineStr">
         <is>
-          <t>현대로템</t>
+          <t>두산퓨얼셀</t>
         </is>
       </c>
       <c r="E27" s="17" t="n">
-        <v>6133.97</v>
+        <v>5907.51</v>
       </c>
       <c r="F27" s="18" t="n">
         <v>2</v>
@@ -1247,23 +1247,23 @@
     </row>
     <row r="28">
       <c r="A28" s="14" t="n">
-        <v>45947</v>
+        <v>45957</v>
       </c>
       <c r="B28" s="14" t="n">
-        <v>45949</v>
+        <v>45959</v>
       </c>
       <c r="C28" s="15" t="inlineStr">
         <is>
-          <t>000150</t>
+          <t>000720</t>
         </is>
       </c>
       <c r="D28" s="16" t="inlineStr">
         <is>
-          <t>두산</t>
+          <t>현대건설</t>
         </is>
       </c>
       <c r="E28" s="17" t="n">
-        <v>5742.17</v>
+        <v>7859.2</v>
       </c>
       <c r="F28" s="18" t="n">
         <v>2</v>
@@ -1271,23 +1271,23 @@
     </row>
     <row r="29">
       <c r="A29" s="14" t="n">
-        <v>45916</v>
+        <v>45650</v>
       </c>
       <c r="B29" s="14" t="n">
-        <v>45945</v>
+        <v>45957</v>
       </c>
       <c r="C29" s="15" t="inlineStr">
         <is>
-          <t>125490</t>
+          <t>196170</t>
         </is>
       </c>
       <c r="D29" s="16" t="inlineStr">
         <is>
-          <t>한라캐스트</t>
+          <t>알테오젠</t>
         </is>
       </c>
       <c r="E29" s="17" t="n">
-        <v>5614.12</v>
+        <v>6894.2</v>
       </c>
       <c r="F29" s="18" t="n">
         <v>2</v>
@@ -1295,119 +1295,119 @@
     </row>
     <row r="30">
       <c r="A30" s="14" t="n">
-        <v>45960</v>
+        <v>45876</v>
       </c>
       <c r="B30" s="14" t="n">
-        <v>45960</v>
+        <v>45957</v>
       </c>
       <c r="C30" s="15" t="inlineStr">
         <is>
-          <t>000270</t>
+          <t>097230</t>
         </is>
       </c>
       <c r="D30" s="16" t="inlineStr">
         <is>
-          <t>기아</t>
+          <t>HJ중공업</t>
         </is>
       </c>
       <c r="E30" s="17" t="n">
-        <v>5648.01</v>
+        <v>6016.41</v>
       </c>
       <c r="F30" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="14" t="n">
-        <v>45959</v>
+        <v>45694</v>
       </c>
       <c r="B31" s="14" t="n">
-        <v>45959</v>
+        <v>45952</v>
       </c>
       <c r="C31" s="15" t="inlineStr">
         <is>
-          <t>001440</t>
+          <t>064350</t>
         </is>
       </c>
       <c r="D31" s="16" t="inlineStr">
         <is>
-          <t>대한전선</t>
+          <t>현대로템</t>
         </is>
       </c>
       <c r="E31" s="17" t="n">
-        <v>5087.57</v>
+        <v>6133.97</v>
       </c>
       <c r="F31" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="14" t="n">
-        <v>45958</v>
+        <v>45947</v>
       </c>
       <c r="B32" s="14" t="n">
-        <v>45958</v>
+        <v>45949</v>
       </c>
       <c r="C32" s="15" t="inlineStr">
         <is>
-          <t>011790</t>
+          <t>000150</t>
         </is>
       </c>
       <c r="D32" s="16" t="inlineStr">
         <is>
-          <t>SKC</t>
+          <t>두산</t>
         </is>
       </c>
       <c r="E32" s="17" t="n">
-        <v>5001.6</v>
+        <v>5742.17</v>
       </c>
       <c r="F32" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="14" t="n">
-        <v>45957</v>
+        <v>45916</v>
       </c>
       <c r="B33" s="14" t="n">
-        <v>45957</v>
+        <v>45945</v>
       </c>
       <c r="C33" s="15" t="inlineStr">
         <is>
-          <t>128940</t>
+          <t>125490</t>
         </is>
       </c>
       <c r="D33" s="16" t="inlineStr">
         <is>
-          <t>한미약품</t>
+          <t>한라캐스트</t>
         </is>
       </c>
       <c r="E33" s="17" t="n">
-        <v>7324.5</v>
+        <v>5614.12</v>
       </c>
       <c r="F33" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="14" t="n">
-        <v>45957</v>
+        <v>45963</v>
       </c>
       <c r="B34" s="14" t="n">
-        <v>45957</v>
+        <v>45963</v>
       </c>
       <c r="C34" s="15" t="inlineStr">
         <is>
-          <t>352820</t>
+          <t>307950</t>
         </is>
       </c>
       <c r="D34" s="16" t="inlineStr">
         <is>
-          <t>하이브</t>
+          <t>현대오토에버</t>
         </is>
       </c>
       <c r="E34" s="17" t="n">
-        <v>5473.690000000001</v>
+        <v>5606.63</v>
       </c>
       <c r="F34" s="18" t="n">
         <v>1</v>
@@ -1415,23 +1415,23 @@
     </row>
     <row r="35">
       <c r="A35" s="14" t="n">
-        <v>45951</v>
+        <v>45958</v>
       </c>
       <c r="B35" s="14" t="n">
-        <v>45951</v>
+        <v>45958</v>
       </c>
       <c r="C35" s="15" t="inlineStr">
         <is>
-          <t>090710</t>
+          <t>011790</t>
         </is>
       </c>
       <c r="D35" s="16" t="inlineStr">
         <is>
-          <t>휴림로봇</t>
+          <t>SKC</t>
         </is>
       </c>
       <c r="E35" s="17" t="n">
-        <v>7343.57</v>
+        <v>5001.6</v>
       </c>
       <c r="F35" s="18" t="n">
         <v>1</v>
@@ -1439,23 +1439,23 @@
     </row>
     <row r="36">
       <c r="A36" s="14" t="n">
-        <v>45943</v>
+        <v>45957</v>
       </c>
       <c r="B36" s="14" t="n">
-        <v>45943</v>
+        <v>45957</v>
       </c>
       <c r="C36" s="15" t="inlineStr">
         <is>
-          <t>466100</t>
+          <t>128940</t>
         </is>
       </c>
       <c r="D36" s="16" t="inlineStr">
         <is>
-          <t>클로봇</t>
+          <t>한미약품</t>
         </is>
       </c>
       <c r="E36" s="17" t="n">
-        <v>6494.860000000001</v>
+        <v>7324.5</v>
       </c>
       <c r="F36" s="18" t="n">
         <v>1</v>
@@ -1463,23 +1463,23 @@
     </row>
     <row r="37">
       <c r="A37" s="14" t="n">
-        <v>44512</v>
+        <v>45957</v>
       </c>
       <c r="B37" s="14" t="n">
-        <v>45929</v>
+        <v>45957</v>
       </c>
       <c r="C37" s="15" t="inlineStr">
         <is>
-          <t>249420</t>
+          <t>352820</t>
         </is>
       </c>
       <c r="D37" s="16" t="inlineStr">
         <is>
-          <t>일동제약</t>
+          <t>하이브</t>
         </is>
       </c>
       <c r="E37" s="17" t="n">
-        <v>9183</v>
+        <v>5473.690000000001</v>
       </c>
       <c r="F37" s="18" t="n">
         <v>1</v>
@@ -1487,23 +1487,23 @@
     </row>
     <row r="38">
       <c r="A38" s="14" t="n">
-        <v>45849</v>
+        <v>45951</v>
       </c>
       <c r="B38" s="14" t="n">
-        <v>45929</v>
+        <v>45951</v>
       </c>
       <c r="C38" s="15" t="inlineStr">
         <is>
-          <t>041190</t>
+          <t>090710</t>
         </is>
       </c>
       <c r="D38" s="16" t="inlineStr">
         <is>
-          <t>우리기술투자</t>
+          <t>휴림로봇</t>
         </is>
       </c>
       <c r="E38" s="17" t="n">
-        <v>5517</v>
+        <v>7343.57</v>
       </c>
       <c r="F38" s="18" t="n">
         <v>1</v>
@@ -1511,23 +1511,23 @@
     </row>
     <row r="39">
       <c r="A39" s="14" t="n">
-        <v>45849</v>
+        <v>45943</v>
       </c>
       <c r="B39" s="14" t="n">
-        <v>45926</v>
+        <v>45943</v>
       </c>
       <c r="C39" s="15" t="inlineStr">
         <is>
-          <t>060250</t>
+          <t>466100</t>
         </is>
       </c>
       <c r="D39" s="16" t="inlineStr">
         <is>
-          <t>NHN KCP</t>
+          <t>클로봇</t>
         </is>
       </c>
       <c r="E39" s="17" t="n">
-        <v>9171</v>
+        <v>6494.860000000001</v>
       </c>
       <c r="F39" s="18" t="n">
         <v>1</v>
@@ -1535,23 +1535,23 @@
     </row>
     <row r="40">
       <c r="A40" s="14" t="n">
-        <v>45925</v>
+        <v>44512</v>
       </c>
       <c r="B40" s="14" t="n">
-        <v>45925</v>
+        <v>45929</v>
       </c>
       <c r="C40" s="15" t="inlineStr">
         <is>
-          <t>277810</t>
+          <t>249420</t>
         </is>
       </c>
       <c r="D40" s="16" t="inlineStr">
         <is>
-          <t>레인보우로보틱스</t>
+          <t>일동제약</t>
         </is>
       </c>
       <c r="E40" s="17" t="n">
-        <v>7211</v>
+        <v>9183</v>
       </c>
       <c r="F40" s="18" t="n">
         <v>1</v>
@@ -1559,23 +1559,23 @@
     </row>
     <row r="41">
       <c r="A41" s="14" t="n">
-        <v>44515</v>
+        <v>45849</v>
       </c>
       <c r="B41" s="14" t="n">
-        <v>45923</v>
+        <v>45929</v>
       </c>
       <c r="C41" s="15" t="inlineStr">
         <is>
-          <t>068270</t>
+          <t>041190</t>
         </is>
       </c>
       <c r="D41" s="16" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>우리기술투자</t>
         </is>
       </c>
       <c r="E41" s="17" t="n">
-        <v>5000</v>
+        <v>5517</v>
       </c>
       <c r="F41" s="18" t="n">
         <v>1</v>
@@ -1583,23 +1583,23 @@
     </row>
     <row r="42">
       <c r="A42" s="14" t="n">
-        <v>45922</v>
+        <v>45849</v>
       </c>
       <c r="B42" s="14" t="n">
-        <v>45923</v>
+        <v>45926</v>
       </c>
       <c r="C42" s="15" t="inlineStr">
         <is>
-          <t>347850</t>
+          <t>060250</t>
         </is>
       </c>
       <c r="D42" s="16" t="inlineStr">
         <is>
-          <t>디앤디파마텍</t>
+          <t>NHN KCP</t>
         </is>
       </c>
       <c r="E42" s="17" t="n">
-        <v>5000</v>
+        <v>9171</v>
       </c>
       <c r="F42" s="18" t="n">
         <v>1</v>
@@ -1607,19 +1607,19 @@
     </row>
     <row r="43">
       <c r="A43" s="14" t="n">
-        <v>45377</v>
+        <v>44515</v>
       </c>
       <c r="B43" s="14" t="n">
-        <v>45919</v>
+        <v>45923</v>
       </c>
       <c r="C43" s="15" t="inlineStr">
         <is>
-          <t>000250</t>
+          <t>068270</t>
         </is>
       </c>
       <c r="D43" s="16" t="inlineStr">
         <is>
-          <t>삼천당제약</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="E43" s="17" t="n">
@@ -1631,19 +1631,19 @@
     </row>
     <row r="44">
       <c r="A44" s="14" t="n">
-        <v>45839</v>
+        <v>45377</v>
       </c>
       <c r="B44" s="14" t="n">
         <v>45919</v>
       </c>
       <c r="C44" s="15" t="inlineStr">
         <is>
-          <t>064260</t>
+          <t>000250</t>
         </is>
       </c>
       <c r="D44" s="16" t="inlineStr">
         <is>
-          <t>다날</t>
+          <t>삼천당제약</t>
         </is>
       </c>
       <c r="E44" s="17" t="n">
@@ -1655,19 +1655,19 @@
     </row>
     <row r="45">
       <c r="A45" s="14" t="n">
-        <v>45918</v>
+        <v>45839</v>
       </c>
       <c r="B45" s="14" t="n">
         <v>45919</v>
       </c>
       <c r="C45" s="15" t="inlineStr">
         <is>
-          <t>090360</t>
+          <t>064260</t>
         </is>
       </c>
       <c r="D45" s="16" t="inlineStr">
         <is>
-          <t>로보스타</t>
+          <t>다날</t>
         </is>
       </c>
       <c r="E45" s="17" t="n">
@@ -1679,19 +1679,19 @@
     </row>
     <row r="46">
       <c r="A46" s="14" t="n">
-        <v>45708</v>
+        <v>45918</v>
       </c>
       <c r="B46" s="14" t="n">
         <v>45919</v>
       </c>
       <c r="C46" s="15" t="inlineStr">
         <is>
-          <t>047810</t>
+          <t>090360</t>
         </is>
       </c>
       <c r="D46" s="16" t="inlineStr">
         <is>
-          <t>한국항공우주</t>
+          <t>로보스타</t>
         </is>
       </c>
       <c r="E46" s="17" t="n">
@@ -1703,19 +1703,19 @@
     </row>
     <row r="47">
       <c r="A47" s="14" t="n">
-        <v>45883</v>
+        <v>45708</v>
       </c>
       <c r="B47" s="14" t="n">
-        <v>45912</v>
+        <v>45919</v>
       </c>
       <c r="C47" s="15" t="inlineStr">
         <is>
-          <t>456160</t>
+          <t>047810</t>
         </is>
       </c>
       <c r="D47" s="16" t="inlineStr">
         <is>
-          <t>지투지바이오</t>
+          <t>한국항공우주</t>
         </is>
       </c>
       <c r="E47" s="17" t="n">
@@ -1727,19 +1727,19 @@
     </row>
     <row r="48">
       <c r="A48" s="14" t="n">
-        <v>45912</v>
+        <v>45883</v>
       </c>
       <c r="B48" s="14" t="n">
         <v>45912</v>
       </c>
       <c r="C48" s="15" t="inlineStr">
         <is>
-          <t>004370</t>
+          <t>456160</t>
         </is>
       </c>
       <c r="D48" s="16" t="inlineStr">
         <is>
-          <t>농심</t>
+          <t>지투지바이오</t>
         </is>
       </c>
       <c r="E48" s="17" t="n">
@@ -1751,19 +1751,19 @@
     </row>
     <row r="49">
       <c r="A49" s="14" t="n">
-        <v>45911</v>
+        <v>45912</v>
       </c>
       <c r="B49" s="14" t="n">
         <v>45912</v>
       </c>
       <c r="C49" s="15" t="inlineStr">
         <is>
-          <t>100090</t>
+          <t>004370</t>
         </is>
       </c>
       <c r="D49" s="16" t="inlineStr">
         <is>
-          <t>SK오션플랜트</t>
+          <t>농심</t>
         </is>
       </c>
       <c r="E49" s="17" t="n">
@@ -1775,19 +1775,19 @@
     </row>
     <row r="50">
       <c r="A50" s="14" t="n">
-        <v>45908</v>
+        <v>45911</v>
       </c>
       <c r="B50" s="14" t="n">
-        <v>45910</v>
+        <v>45912</v>
       </c>
       <c r="C50" s="15" t="inlineStr">
         <is>
-          <t>075580</t>
+          <t>100090</t>
         </is>
       </c>
       <c r="D50" s="16" t="inlineStr">
         <is>
-          <t>세진중공업</t>
+          <t>SK오션플랜트</t>
         </is>
       </c>
       <c r="E50" s="17" t="n">
@@ -1802,16 +1802,16 @@
         <v>45908</v>
       </c>
       <c r="B51" s="14" t="n">
-        <v>45908</v>
+        <v>45910</v>
       </c>
       <c r="C51" s="15" t="inlineStr">
         <is>
-          <t>290650</t>
+          <t>075580</t>
         </is>
       </c>
       <c r="D51" s="16" t="inlineStr">
         <is>
-          <t>엘앤씨바이오</t>
+          <t>세진중공업</t>
         </is>
       </c>
       <c r="E51" s="17" t="n">
@@ -1823,19 +1823,19 @@
     </row>
     <row r="52">
       <c r="A52" s="14" t="n">
-        <v>45898</v>
+        <v>45908</v>
       </c>
       <c r="B52" s="14" t="n">
-        <v>45898</v>
+        <v>45908</v>
       </c>
       <c r="C52" s="15" t="inlineStr">
         <is>
-          <t>082740</t>
+          <t>290650</t>
         </is>
       </c>
       <c r="D52" s="16" t="inlineStr">
         <is>
-          <t>한화엔진</t>
+          <t>엘앤씨바이오</t>
         </is>
       </c>
       <c r="E52" s="17" t="n">
@@ -1847,19 +1847,19 @@
     </row>
     <row r="53">
       <c r="A53" s="14" t="n">
-        <v>45897</v>
+        <v>45898</v>
       </c>
       <c r="B53" s="14" t="n">
-        <v>45897</v>
+        <v>45898</v>
       </c>
       <c r="C53" s="15" t="inlineStr">
         <is>
-          <t>460930</t>
+          <t>082740</t>
         </is>
       </c>
       <c r="D53" s="16" t="inlineStr">
         <is>
-          <t>현대힘스</t>
+          <t>한화엔진</t>
         </is>
       </c>
       <c r="E53" s="17" t="n">
@@ -1878,12 +1878,12 @@
       </c>
       <c r="C54" s="15" t="inlineStr">
         <is>
-          <t>009540</t>
+          <t>460930</t>
         </is>
       </c>
       <c r="D54" s="16" t="inlineStr">
         <is>
-          <t>HD한국조선해양</t>
+          <t>현대힘스</t>
         </is>
       </c>
       <c r="E54" s="17" t="n">
@@ -1895,19 +1895,19 @@
     </row>
     <row r="55">
       <c r="A55" s="14" t="n">
-        <v>45896</v>
+        <v>45897</v>
       </c>
       <c r="B55" s="14" t="n">
         <v>45897</v>
       </c>
       <c r="C55" s="15" t="inlineStr">
         <is>
-          <t>010620</t>
+          <t>009540</t>
         </is>
       </c>
       <c r="D55" s="16" t="inlineStr">
         <is>
-          <t>HD현대미포</t>
+          <t>HD한국조선해양</t>
         </is>
       </c>
       <c r="E55" s="17" t="n">
@@ -1919,19 +1919,19 @@
     </row>
     <row r="56">
       <c r="A56" s="14" t="n">
-        <v>45895</v>
+        <v>45896</v>
       </c>
       <c r="B56" s="14" t="n">
-        <v>45895</v>
+        <v>45897</v>
       </c>
       <c r="C56" s="15" t="inlineStr">
         <is>
-          <t>298040</t>
+          <t>010620</t>
         </is>
       </c>
       <c r="D56" s="16" t="inlineStr">
         <is>
-          <t>효성중공업</t>
+          <t>HD현대미포</t>
         </is>
       </c>
       <c r="E56" s="17" t="n">
@@ -1943,19 +1943,19 @@
     </row>
     <row r="57">
       <c r="A57" s="14" t="n">
-        <v>45782</v>
+        <v>45895</v>
       </c>
       <c r="B57" s="14" t="n">
         <v>45895</v>
       </c>
       <c r="C57" s="15" t="inlineStr">
         <is>
-          <t>079550</t>
+          <t>298040</t>
         </is>
       </c>
       <c r="D57" s="16" t="inlineStr">
         <is>
-          <t>LIG넥스원</t>
+          <t>효성중공업</t>
         </is>
       </c>
       <c r="E57" s="17" t="n">
@@ -1967,19 +1967,19 @@
     </row>
     <row r="58">
       <c r="A58" s="14" t="n">
-        <v>45888</v>
+        <v>45782</v>
       </c>
       <c r="B58" s="14" t="n">
-        <v>45888</v>
+        <v>45895</v>
       </c>
       <c r="C58" s="15" t="inlineStr">
         <is>
-          <t>0008Z0</t>
+          <t>079550</t>
         </is>
       </c>
       <c r="D58" s="16" t="inlineStr">
         <is>
-          <t>에스엔시스</t>
+          <t>LIG넥스원</t>
         </is>
       </c>
       <c r="E58" s="17" t="n">
@@ -1991,19 +1991,19 @@
     </row>
     <row r="59">
       <c r="A59" s="14" t="n">
-        <v>45887</v>
+        <v>45888</v>
       </c>
       <c r="B59" s="14" t="n">
-        <v>45887</v>
+        <v>45888</v>
       </c>
       <c r="C59" s="15" t="inlineStr">
         <is>
-          <t>484590</t>
+          <t>0008Z0</t>
         </is>
       </c>
       <c r="D59" s="16" t="inlineStr">
         <is>
-          <t>삼양컴텍</t>
+          <t>에스엔시스</t>
         </is>
       </c>
       <c r="E59" s="17" t="n">
@@ -2015,19 +2015,19 @@
     </row>
     <row r="60">
       <c r="A60" s="14" t="n">
-        <v>45755</v>
+        <v>45887</v>
       </c>
       <c r="B60" s="14" t="n">
-        <v>45883</v>
+        <v>45887</v>
       </c>
       <c r="C60" s="15" t="inlineStr">
         <is>
-          <t>298380</t>
+          <t>484590</t>
         </is>
       </c>
       <c r="D60" s="16" t="inlineStr">
         <is>
-          <t>에이비엘바이오</t>
+          <t>삼양컴텍</t>
         </is>
       </c>
       <c r="E60" s="17" t="n">
@@ -2039,19 +2039,19 @@
     </row>
     <row r="61">
       <c r="A61" s="14" t="n">
-        <v>45882</v>
+        <v>45755</v>
       </c>
       <c r="B61" s="14" t="n">
-        <v>45882</v>
+        <v>45883</v>
       </c>
       <c r="C61" s="15" t="inlineStr">
         <is>
-          <t>034220</t>
+          <t>298380</t>
         </is>
       </c>
       <c r="D61" s="16" t="inlineStr">
         <is>
-          <t>LG디스플레이</t>
+          <t>에이비엘바이오</t>
         </is>
       </c>
       <c r="E61" s="17" t="n">
@@ -2063,19 +2063,19 @@
     </row>
     <row r="62">
       <c r="A62" s="14" t="n">
-        <v>45870</v>
+        <v>45882</v>
       </c>
       <c r="B62" s="14" t="n">
-        <v>45876</v>
+        <v>45882</v>
       </c>
       <c r="C62" s="15" t="inlineStr">
         <is>
-          <t>439260</t>
+          <t>034220</t>
         </is>
       </c>
       <c r="D62" s="16" t="inlineStr">
         <is>
-          <t>대한조선</t>
+          <t>LG디스플레이</t>
         </is>
       </c>
       <c r="E62" s="17" t="n">
@@ -2087,19 +2087,19 @@
     </row>
     <row r="63">
       <c r="A63" s="14" t="n">
-        <v>45785</v>
+        <v>45870</v>
       </c>
       <c r="B63" s="14" t="n">
-        <v>45875</v>
+        <v>45876</v>
       </c>
       <c r="C63" s="15" t="inlineStr">
         <is>
-          <t>278470</t>
+          <t>439260</t>
         </is>
       </c>
       <c r="D63" s="16" t="inlineStr">
         <is>
-          <t>에이피알</t>
+          <t>대한조선</t>
         </is>
       </c>
       <c r="E63" s="17" t="n">
@@ -2111,19 +2111,19 @@
     </row>
     <row r="64">
       <c r="A64" s="14" t="n">
-        <v>45874</v>
+        <v>45785</v>
       </c>
       <c r="B64" s="14" t="n">
-        <v>45874</v>
+        <v>45875</v>
       </c>
       <c r="C64" s="15" t="inlineStr">
         <is>
-          <t>326030</t>
+          <t>278470</t>
         </is>
       </c>
       <c r="D64" s="16" t="inlineStr">
         <is>
-          <t>SK바이오팜</t>
+          <t>에이피알</t>
         </is>
       </c>
       <c r="E64" s="17" t="n">
@@ -2135,19 +2135,19 @@
     </row>
     <row r="65">
       <c r="A65" s="14" t="n">
-        <v>45699</v>
+        <v>45874</v>
       </c>
       <c r="B65" s="14" t="n">
-        <v>45870</v>
+        <v>45874</v>
       </c>
       <c r="C65" s="15" t="inlineStr">
         <is>
-          <t>012450</t>
+          <t>326030</t>
         </is>
       </c>
       <c r="D65" s="16" t="inlineStr">
         <is>
-          <t>한화에어로스페이스</t>
+          <t>SK바이오팜</t>
         </is>
       </c>
       <c r="E65" s="17" t="n">
@@ -2159,19 +2159,19 @@
     </row>
     <row r="66">
       <c r="A66" s="14" t="n">
-        <v>45772</v>
+        <v>45699</v>
       </c>
       <c r="B66" s="14" t="n">
-        <v>45868</v>
+        <v>45870</v>
       </c>
       <c r="C66" s="15" t="inlineStr">
         <is>
-          <t>009830</t>
+          <t>012450</t>
         </is>
       </c>
       <c r="D66" s="16" t="inlineStr">
         <is>
-          <t>한화솔루션</t>
+          <t>한화에어로스페이스</t>
         </is>
       </c>
       <c r="E66" s="17" t="n">
@@ -2183,19 +2183,19 @@
     </row>
     <row r="67">
       <c r="A67" s="14" t="n">
-        <v>45868</v>
+        <v>45772</v>
       </c>
       <c r="B67" s="14" t="n">
         <v>45868</v>
       </c>
       <c r="C67" s="15" t="inlineStr">
         <is>
-          <t>009150</t>
+          <t>009830</t>
         </is>
       </c>
       <c r="D67" s="16" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>한화솔루션</t>
         </is>
       </c>
       <c r="E67" s="17" t="n">
@@ -2207,19 +2207,19 @@
     </row>
     <row r="68">
       <c r="A68" s="14" t="n">
-        <v>45867</v>
+        <v>45868</v>
       </c>
       <c r="B68" s="14" t="n">
-        <v>45867</v>
+        <v>45868</v>
       </c>
       <c r="C68" s="15" t="inlineStr">
         <is>
-          <t>489790</t>
+          <t>009150</t>
         </is>
       </c>
       <c r="D68" s="16" t="inlineStr">
         <is>
-          <t>한화비전</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="E68" s="17" t="n">
@@ -2231,19 +2231,19 @@
     </row>
     <row r="69">
       <c r="A69" s="14" t="n">
-        <v>45862</v>
+        <v>45867</v>
       </c>
       <c r="B69" s="14" t="n">
         <v>45867</v>
       </c>
       <c r="C69" s="15" t="inlineStr">
         <is>
-          <t>042670</t>
+          <t>489790</t>
         </is>
       </c>
       <c r="D69" s="16" t="inlineStr">
         <is>
-          <t>HD현대인프라코어</t>
+          <t>한화비전</t>
         </is>
       </c>
       <c r="E69" s="17" t="n">
@@ -2255,19 +2255,19 @@
     </row>
     <row r="70">
       <c r="A70" s="14" t="n">
-        <v>45861</v>
+        <v>45862</v>
       </c>
       <c r="B70" s="14" t="n">
-        <v>45861</v>
+        <v>45867</v>
       </c>
       <c r="C70" s="15" t="inlineStr">
         <is>
-          <t>484120</t>
+          <t>042670</t>
         </is>
       </c>
       <c r="D70" s="16" t="inlineStr">
         <is>
-          <t>도우인시스</t>
+          <t>HD현대인프라코어</t>
         </is>
       </c>
       <c r="E70" s="17" t="n">
@@ -2279,19 +2279,19 @@
     </row>
     <row r="71">
       <c r="A71" s="14" t="n">
-        <v>45846</v>
+        <v>45861</v>
       </c>
       <c r="B71" s="14" t="n">
         <v>45861</v>
       </c>
       <c r="C71" s="15" t="inlineStr">
         <is>
-          <t>008970</t>
+          <t>484120</t>
         </is>
       </c>
       <c r="D71" s="16" t="inlineStr">
         <is>
-          <t>KBI동양철관</t>
+          <t>도우인시스</t>
         </is>
       </c>
       <c r="E71" s="17" t="n">
@@ -2303,19 +2303,19 @@
     </row>
     <row r="72">
       <c r="A72" s="14" t="n">
-        <v>45860</v>
+        <v>45846</v>
       </c>
       <c r="B72" s="14" t="n">
-        <v>45860</v>
+        <v>45861</v>
       </c>
       <c r="C72" s="15" t="inlineStr">
         <is>
-          <t>037270</t>
+          <t>008970</t>
         </is>
       </c>
       <c r="D72" s="16" t="inlineStr">
         <is>
-          <t>YG PLUS</t>
+          <t>KBI동양철관</t>
         </is>
       </c>
       <c r="E72" s="17" t="n">
@@ -2327,19 +2327,19 @@
     </row>
     <row r="73">
       <c r="A73" s="14" t="n">
-        <v>45856</v>
+        <v>45860</v>
       </c>
       <c r="B73" s="14" t="n">
-        <v>45856</v>
+        <v>45860</v>
       </c>
       <c r="C73" s="15" t="inlineStr">
         <is>
-          <t>141080</t>
+          <t>037270</t>
         </is>
       </c>
       <c r="D73" s="16" t="inlineStr">
         <is>
-          <t>리가켐바이오</t>
+          <t>YG PLUS</t>
         </is>
       </c>
       <c r="E73" s="17" t="n">
@@ -2351,19 +2351,19 @@
     </row>
     <row r="74">
       <c r="A74" s="14" t="n">
-        <v>45854</v>
+        <v>45856</v>
       </c>
       <c r="B74" s="14" t="n">
-        <v>45854</v>
+        <v>45856</v>
       </c>
       <c r="C74" s="15" t="inlineStr">
         <is>
-          <t>294570</t>
+          <t>141080</t>
         </is>
       </c>
       <c r="D74" s="16" t="inlineStr">
         <is>
-          <t>쿠콘</t>
+          <t>리가켐바이오</t>
         </is>
       </c>
       <c r="E74" s="17" t="n">
@@ -2382,12 +2382,12 @@
       </c>
       <c r="C75" s="15" t="inlineStr">
         <is>
-          <t>441270</t>
+          <t>294570</t>
         </is>
       </c>
       <c r="D75" s="16" t="inlineStr">
         <is>
-          <t>파인엠텍</t>
+          <t>쿠콘</t>
         </is>
       </c>
       <c r="E75" s="17" t="n">
@@ -2399,19 +2399,19 @@
     </row>
     <row r="76">
       <c r="A76" s="14" t="n">
-        <v>45849</v>
+        <v>45854</v>
       </c>
       <c r="B76" s="14" t="n">
-        <v>45849</v>
+        <v>45854</v>
       </c>
       <c r="C76" s="15" t="inlineStr">
         <is>
-          <t>402340</t>
+          <t>441270</t>
         </is>
       </c>
       <c r="D76" s="16" t="inlineStr">
         <is>
-          <t>SK스퀘어</t>
+          <t>파인엠텍</t>
         </is>
       </c>
       <c r="E76" s="17" t="n">
@@ -2423,19 +2423,19 @@
     </row>
     <row r="77">
       <c r="A77" s="14" t="n">
-        <v>45841</v>
+        <v>45849</v>
       </c>
       <c r="B77" s="14" t="n">
-        <v>45842</v>
+        <v>45849</v>
       </c>
       <c r="C77" s="15" t="inlineStr">
         <is>
-          <t>005490</t>
+          <t>402340</t>
         </is>
       </c>
       <c r="D77" s="16" t="inlineStr">
         <is>
-          <t>POSCO홀딩스</t>
+          <t>SK스퀘어</t>
         </is>
       </c>
       <c r="E77" s="17" t="n">
@@ -2447,19 +2447,19 @@
     </row>
     <row r="78">
       <c r="A78" s="14" t="n">
-        <v>45840</v>
+        <v>45841</v>
       </c>
       <c r="B78" s="14" t="n">
-        <v>45840</v>
+        <v>45842</v>
       </c>
       <c r="C78" s="15" t="inlineStr">
         <is>
-          <t>267270</t>
+          <t>005490</t>
         </is>
       </c>
       <c r="D78" s="16" t="inlineStr">
         <is>
-          <t>HD현대건설기계</t>
+          <t>POSCO홀딩스</t>
         </is>
       </c>
       <c r="E78" s="17" t="n">
@@ -2471,19 +2471,19 @@
     </row>
     <row r="79">
       <c r="A79" s="14" t="n">
-        <v>45839</v>
+        <v>45840</v>
       </c>
       <c r="B79" s="14" t="n">
-        <v>45839</v>
+        <v>45840</v>
       </c>
       <c r="C79" s="15" t="inlineStr">
         <is>
-          <t>000880</t>
+          <t>267270</t>
         </is>
       </c>
       <c r="D79" s="16" t="inlineStr">
         <is>
-          <t>한화</t>
+          <t>HD현대건설기계</t>
         </is>
       </c>
       <c r="E79" s="17" t="n">
@@ -2495,19 +2495,19 @@
     </row>
     <row r="80">
       <c r="A80" s="14" t="n">
-        <v>43997</v>
+        <v>45839</v>
       </c>
       <c r="B80" s="14" t="n">
         <v>45839</v>
       </c>
       <c r="C80" s="15" t="inlineStr">
         <is>
-          <t>034730</t>
+          <t>000880</t>
         </is>
       </c>
       <c r="D80" s="16" t="inlineStr">
         <is>
-          <t>SK</t>
+          <t>한화</t>
         </is>
       </c>
       <c r="E80" s="17" t="n">
@@ -2519,25 +2519,49 @@
     </row>
     <row r="81">
       <c r="A81" s="14" t="n">
-        <v>45838</v>
+        <v>43997</v>
       </c>
       <c r="B81" s="14" t="n">
         <v>45839</v>
       </c>
       <c r="C81" s="15" t="inlineStr">
         <is>
+          <t>034730</t>
+        </is>
+      </c>
+      <c r="D81" s="16" t="inlineStr">
+        <is>
+          <t>SK</t>
+        </is>
+      </c>
+      <c r="E81" s="17" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F81" s="18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="14" t="n">
+        <v>45838</v>
+      </c>
+      <c r="B82" s="14" t="n">
+        <v>45839</v>
+      </c>
+      <c r="C82" s="15" t="inlineStr">
+        <is>
           <t>096770</t>
         </is>
       </c>
-      <c r="D81" s="16" t="inlineStr">
+      <c r="D82" s="16" t="inlineStr">
         <is>
           <t>SK이노베이션</t>
         </is>
       </c>
-      <c r="E81" s="17" t="n">
-        <v>5000</v>
-      </c>
-      <c r="F81" s="18" t="n">
+      <c r="E82" s="17" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F82" s="18" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>